<commit_message>
some changes in backend
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -1343,1043 +1343,1043 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Erik Bernhardsson</t>
+          <t>Jarrod Gingras</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Real Story Group</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>Managing Director &amp; DAM Analyst</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Real Story Group</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Modal founder &amp; CEO; pioneer in serverless container runtimes, GPU virtualization, and distributed systems. Keynotes at PyData, Strange Loop, MLSys.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Will Reese</t>
+          <t>Mike Szumlinski</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Backlight</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Founding Engineer &amp; Systems Architect</t>
+          <t>Field Chief Technology Officer</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Backlight</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Modal founding engineer specializing in microVM architecture, Linux cgroups, and high-throughput container virtualization.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Akshat Bubna</t>
+          <t>John Horodyski</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Salt Flats</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>AI Infrastructure Lead</t>
+          <t>Executive Director, Information &amp; Data Strategy</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Salt Flats</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Modal engineering lead for distributed GPU inference, model sharding, and cluster auto-scaling.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Jonathon Belotti</t>
+          <t>Theresa Regli</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Independent Consultant</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Staff Systems Engineer</t>
+          <t>Digital Asset Strategist &amp; Author</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Independent Consultant</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Boston, MA, USA</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Systems architect for distributed execution engines, low-latency microVM architecture, and edge runtimes.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Charles Fry</t>
+          <t>Graham Allan</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>The Home Depot</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Distributed Systems Lead</t>
+          <t>Senior Manager, Content Architecture &amp; DAM</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>The Home Depot</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Atlanta, GA, USA</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Cloud infrastructure architect; speaker on large-scale cluster orchestration and resilient workload scheduling.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Luis Ceze</t>
+          <t>David Lipsey</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>University of Washington &amp; OctoAI</t>
+          <t>The DAM Foundation</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>CEO &amp; Professor of Computer Science</t>
+          <t>Chair</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>University of Washington &amp; OctoAI</t>
+          <t>The DAM Foundation</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Seattle, WA, USA</t>
+          <t>Philadelphia, PA, USA</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>UW Professor &amp; OctoAI CEO; keynote speaker at ASPLOS, ISCA, NeurIPS on hardware-software co-design for AI and efficient deep learning compilation.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Tri Dao</t>
+          <t>Cynthia Simpson</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Together AI &amp; Princeton University</t>
+          <t>The Estée Lauder Companies</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Chief Scientist &amp; Assistant Professor</t>
+          <t>Global DAM &amp; Creative Operations Director</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Together AI &amp; Princeton University</t>
+          <t>The Estée Lauder Companies</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Princeton, NJ, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Creator of FlashAttention; invited speaker at NeurIPS, ICML, MLSys on linear and sub-quadratic attention architectures and kernel optimization.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Horace He</t>
+          <t>Frederic Sanuy</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>PyTorch Core &amp; Meta AI</t>
+          <t>Activo DAM Consulting</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer</t>
+          <t>CEO &amp; Chief Solutions Architect</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>PyTorch Core &amp; Meta AI</t>
+          <t>Activo DAM Consulting</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>PyTorch core engineer; speaker on torch.compile, compiler optimizations, GPU kernel codegen, and tensor program synthesis.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Tim Dettmers</t>
+          <t>Mark Davey</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Allen Institute for AI &amp; University of Washington</t>
+          <t>The CODIFY Group</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Assistant Professor &amp; Research Scientist</t>
+          <t>Founder &amp; Director</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Allen Institute for AI &amp; University of Washington</t>
+          <t>The CODIFY Group</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Seattle, WA, USA</t>
+          <t>London / New York, USA</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Creator of bitsandbytes (8-bit &amp; 4-bit quantization, QLoRA); keynote speaker on efficient deep learning and memory-bounded LLM fine-tuning.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Bert Maher</t>
+          <t>Jennifer Allen</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Meta AI</t>
+          <t>Sony Pictures Entertainment</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Compiler Engineering Lead</t>
+          <t>Director of Global Asset Management &amp; Content Systems</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Meta AI</t>
+          <t>Sony Pictures Entertainment</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Menlo Park, CA, USA</t>
+          <t>Los Angeles, CA, USA</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Meta AI compiler lead; technical talks on deep learning compilers, AOTInductor, and high-performance ML inference backends.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Dan Fu</t>
+          <t>Linda Tadic</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Stanford University &amp; Cartesia</t>
+          <t>Digital Bedrock</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>AI Systems Researcher</t>
+          <t>CEO &amp; Founder</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Stanford University &amp; Cartesia</t>
+          <t>Digital Bedrock</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Stanford, CA, USA</t>
+          <t>Los Angeles, CA, USA</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Co-creator of FlashAttention, H3, and Monarch architectures; speaker on efficient long-context sequence modeling at ICML and MLSys.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Sarah Catanzaro</t>
+          <t>Craig Llewellyn</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Amplify Partners</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>General Partner</t>
+          <t>Director of Enterprise Creative Tech</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Amplify Partners</t>
+          <t>Warner Bros. Discovery</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Keynote speaker on AI infrastructure investing, open-source AI ecosystems, and developer tooling at Scale AI and O'Reilly Strata.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Beidi Chen</t>
+          <t>Ian Matzen</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Carnegie Mellon University</t>
+          <t>NBCUniversal</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Metadata &amp; Taxonomy Lead</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Carnegie Mellon University</t>
+          <t>NBCUniversal</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>CMU faculty; invited speaker on algorithm-hardware co-design for efficient LLM training and inference at MLSys and CVPR.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Greg Brockman</t>
+          <t>Reem El Asaleh</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>DAM New York 2026</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Toronto Metropolitan University</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>President &amp; Co-Founder</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Toronto Metropolitan University</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Toronto / New York, USA</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>OpenAI President &amp; Co-founder; keynote addresses at SXSW, TechCrunch Disrupt, and MIT on scaling laws, supercomputing infrastructure, and frontier AI models.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Sandra Hundacker</t>
+          <t>Erik Bernhardsson</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Rick Steves' Europe</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Creative &amp; Operations Director</t>
+          <t>Founder &amp; CEO</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Rick Steves' Europe</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Edmonds, WA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on enterprise content supply chains, multi-platform media publishing, and automated asset governance at Henry Stewart DAM Europe.</t>
+          <t>Modal founder &amp; CEO; pioneer in serverless container runtimes, GPU virtualization, and distributed systems. Keynotes at PyData, Strange Loop, MLSys.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Orin Dubrow</t>
+          <t>Will Reese</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Rick Steves' Europe</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Creative Operations &amp; Production Specialist</t>
+          <t>Founding Engineer &amp; Systems Architect</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Rick Steves' Europe</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Edmonds, WA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Sessions on digital taxonomy design, multi-channel asset integration, and operational metadata standards.</t>
+          <t>Modal founding engineer specializing in microVM architecture, Linux cgroups, and high-throughput container virtualization.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Jarrod Gingras</t>
+          <t>Akshat Bubna</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Real Story Group</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Managing Director &amp; DAM Analyst</t>
+          <t>AI Infrastructure Lead</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Real Story Group</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Industry keynotes on enterprise DAM vendor landscapes, martech stack evaluation, and headless content architecture at DAM Clinic.</t>
+          <t>Modal engineering lead for distributed GPU inference, model sharding, and cluster auto-scaling.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Mike Szumlinski</t>
+          <t>Jonathon Belotti</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Backlight</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Field Chief Technology Officer</t>
+          <t>Staff Systems Engineer</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Backlight</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Presentations on AI-driven automated metadata tagging, cloud video asset pipelines, and media workflow orchestration at NAB Show.</t>
+          <t>Systems architect for distributed execution engines, low-latency microVM architecture, and edge runtimes.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>John Horodyski</t>
+          <t>Charles Fry</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Salt Flats</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Executive Director, Information &amp; Data Strategy</t>
+          <t>Distributed Systems Lead</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Salt Flats</t>
+          <t>Modal Labs</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Author and keynote speaker on metadata governance, semantic data strategy, and enterprise information taxonomy.</t>
+          <t>Cloud infrastructure architect; speaker on large-scale cluster orchestration and resilient workload scheduling.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Theresa Regli</t>
+          <t>Luis Ceze</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Independent Consultant</t>
+          <t>University of Washington &amp; OctoAI</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Digital Asset Strategist &amp; Author</t>
+          <t>CEO &amp; Professor of Computer Science</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Independent Consultant</t>
+          <t>University of Washington &amp; OctoAI</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Boston, MA, USA</t>
+          <t>Seattle, WA, USA</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Author of "Digital &amp; Marketing Asset Management"; global speaker on content technologies and DAM maturity models.</t>
+          <t>UW Professor &amp; OctoAI CEO; keynote speaker at ASPLOS, ISCA, NeurIPS on hardware-software co-design for AI and efficient deep learning compilation.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Graham Allan</t>
+          <t>Tri Dao</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>The Home Depot</t>
+          <t>Together AI &amp; Princeton University</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Senior Manager, Content Architecture &amp; DAM</t>
+          <t>Chief Scientist &amp; Assistant Professor</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>The Home Depot</t>
+          <t>Together AI &amp; Princeton University</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Atlanta, GA, USA</t>
+          <t>Princeton, NJ, USA</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Presentations on omnichannel retail digital asset supply chains and large-scale enterprise catalog architecture.</t>
+          <t>Creator of FlashAttention; invited speaker at NeurIPS, ICML, MLSys on linear and sub-quadratic attention architectures and kernel optimization.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>David Lipsey</t>
+          <t>Horace He</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>The DAM Foundation</t>
+          <t>PyTorch Core &amp; Meta AI</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Chair</t>
+          <t>Machine Learning Systems Engineer</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>The DAM Foundation</t>
+          <t>PyTorch Core &amp; Meta AI</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Philadelphia, PA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Founding Chair of DAM Foundation; keynote speaker on DAM credentialing, industry standards, and digital rights.</t>
+          <t>PyTorch core engineer; speaker on torch.compile, compiler optimizations, GPU kernel codegen, and tensor program synthesis.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Cynthia Simpson</t>
+          <t>Tim Dettmers</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>The Estée Lauder Companies</t>
+          <t>Allen Institute for AI &amp; University of Washington</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Global DAM &amp; Creative Operations Director</t>
+          <t>Assistant Professor &amp; Research Scientist</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>The Estée Lauder Companies</t>
+          <t>Allen Institute for AI &amp; University of Washington</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>Seattle, WA, USA</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on global prestige beauty brand asset orchestration, rights management, and packaging workflows.</t>
+          <t>Creator of bitsandbytes (8-bit &amp; 4-bit quantization, QLoRA); keynote speaker on efficient deep learning and memory-bounded LLM fine-tuning.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Frederic Sanuy</t>
+          <t>Bert Maher</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Activo DAM Consulting</t>
+          <t>Meta AI</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>CEO &amp; Chief Solutions Architect</t>
+          <t>Compiler Engineering Lead</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Activo DAM Consulting</t>
+          <t>Meta AI</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>Menlo Park, CA, USA</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Speaker on DAM implementation frameworks, European and North American enterprise martech architectures.</t>
+          <t>Meta AI compiler lead; technical talks on deep learning compilers, AOTInductor, and high-performance ML inference backends.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Mark Davey</t>
+          <t>Dan Fu</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>The CODIFY Group</t>
+          <t>Stanford University &amp; Cartesia</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Founder &amp; Director</t>
+          <t>AI Systems Researcher</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>The CODIFY Group</t>
+          <t>Stanford University &amp; Cartesia</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>London / New York, USA</t>
+          <t>Stanford, CA, USA</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Creator of DAM Maturity Model; speaker on digital asset strategy, metadata automation, and vendor benchmarking.</t>
+          <t>Co-creator of FlashAttention, H3, and Monarch architectures; speaker on efficient long-context sequence modeling at ICML and MLSys.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Jennifer Allen</t>
+          <t>Sarah Catanzaro</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Sony Pictures Entertainment</t>
+          <t>Amplify Partners</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Director of Global Asset Management &amp; Content Systems</t>
+          <t>General Partner</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Sony Pictures Entertainment</t>
+          <t>Amplify Partners</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Studio keynote on global film &amp; TV asset distribution, preservation archiving, and digital master workflows.</t>
+          <t>Keynote speaker on AI infrastructure investing, open-source AI ecosystems, and developer tooling at Scale AI and O'Reilly Strata.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Linda Tadic</t>
+          <t>Beidi Chen</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Digital Bedrock</t>
+          <t>Carnegie Mellon University</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>CEO &amp; Founder</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Digital Bedrock</t>
+          <t>Carnegie Mellon University</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, USA</t>
+          <t>Pittsburgh, PA, USA</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Digital preservation authority; keynote speaker at AMIA and SAA on long-term digital media file health and preservation metadata.</t>
+          <t>CMU faculty; invited speaker on algorithm-hardware co-design for efficient LLM training and inference at MLSys and CVPR.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Craig Llewellyn</t>
+          <t>Greg Brockman</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>Runtime by Modal</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Director of Enterprise Creative Tech</t>
+          <t>President &amp; Co-Founder</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Speaker on creative tech toolchains, generative AI in post-production asset systems, and collaborative editing storage.</t>
+          <t>OpenAI President &amp; Co-founder; keynote addresses at SXSW, TechCrunch Disrupt, and MIT on scaling laws, supercomputing infrastructure, and frontier AI models.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Ian Matzen</t>
+          <t>Sandra Hundacker</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -2389,34 +2389,34 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>NBCUniversal</t>
+          <t>Rick Steves' Europe</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Metadata &amp; Taxonomy Lead</t>
+          <t>Creative &amp; Operations Director</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>NBCUniversal</t>
+          <t>Rick Steves' Europe</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>Edmonds, WA, USA</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Presentations on broadcast media metadata schemas, automated speech-to-text tagging, and entertainment metadata workflows.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Reem El Asaleh</t>
+          <t>Orin Dubrow</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -2426,27 +2426,27 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Toronto Metropolitan University</t>
+          <t>Rick Steves' Europe</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Creative Operations &amp; Production Specialist</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Toronto Metropolitan University</t>
+          <t>Rick Steves' Europe</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Toronto / New York, USA</t>
+          <t>Edmonds, WA, USA</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Academic researcher; speaker on color science, digital asset management workflows, and media production systems.</t>
+          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adding a speakers linkedin and company website url
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -459,18 +459,18 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="51" customWidth="1" min="3" max="3"/>
+    <col width="57" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="41" customWidth="1" min="7" max="7"/>
+    <col width="67" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="48" customWidth="1" min="10" max="10"/>
-    <col width="67" customWidth="1" min="11" max="11"/>
-    <col width="67" customWidth="1" min="12" max="12"/>
-    <col width="58" customWidth="1" min="13" max="13"/>
+    <col width="64" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="94" customWidth="1" min="12" max="12"/>
+    <col width="94" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -549,27 +549,27 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>CONF-2026-961D4E</t>
+          <t>CONF-2026-072AD3</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>AASCP Fall Regenerative Medicine Conference Miami 2026</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Cloud Infrastructure &amp; AI Systems</t>
+          <t>Healthcare IT</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>San Francisco Design Center</t>
+          <t>Hyatt Regency Miami, 400 SE 2nd Ave, Miami, FL, USA</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -594,54 +594,54 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs &amp; Luma</t>
+          <t>American Academy of Stem Cell Physicians (AASCP) &amp; Eventbrite</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>https://modal.com</t>
+          <t>https://aascp.net</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>https://lu.ma/runtime-by-modal</t>
+          <t>https://www.eventbrite.com/e/aascp-2026-fall-regenerative-medicine-conference-miami-tickets</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>https://lu.ma/runtime-by-modal</t>
+          <t>https://www.eventbrite.com/e/aascp-2026-fall-regenerative-medicine-conference-miami-tickets</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-06-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CONF-2026-9DFE34</t>
+          <t>CONF-2026-8792EC</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Digital Asset Management &amp; Enterprise AI Systems</t>
+          <t>Cybersecurity &amp; Cloud</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -651,12 +651,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>New York Hilton Midtown</t>
+          <t>RiverCenter, Davenport, Iowa, USA</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Davenport</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -666,54 +666,54 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Henry Stewart Conferences &amp; Eventbrite</t>
+          <t>Docent Institute &amp; CornCon</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>https://www.henrystewartconferences.com/events/dam-new-york-2026</t>
+          <t>https://corncon.net</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>https://www.henrystewartconferences.com/events/dam-new-york-2026</t>
+          <t>https://corncon.net/tickets</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/d/ny--new-york/dam-new-york/</t>
+          <t>https://10times.com/corncon</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CONF-2026-6E1919</t>
+          <t>CONF-2026-EAA412</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Cybersecurity &amp; Cloud Infrastructure</t>
+          <t>Healthcare IT</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Walter E. Washington Convention Center</t>
+          <t>San Diego Convention Center, 111 W Harbor Dr, San Diego, CA, USA</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -738,27 +738,27 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>National Cyber Security Association &amp; 10times</t>
+          <t>American Academy of Pediatrics &amp; Events in America</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>https://cybersecuritysummit.com</t>
+          <t>https://aapexperience.org</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>https://cybersecuritysummit.com</t>
+          <t>https://aapexperience.org/registration</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>https://10times.com/cyber-cloud-security-summit</t>
+          <t>https://eventsinamerica.com/events/aap-national-conference-exhibition-2026</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -773,16 +773,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="69" customWidth="1" min="4" max="4"/>
-    <col width="56" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="230" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="57" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="73" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="51" customWidth="1" min="6" max="6"/>
+    <col width="64" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -813,1640 +814,3981 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
+          <t>Official Company Website URL</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Speaker LinkedIn Profile URL</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Location</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Previous Conference / Event Speaking Information, if available</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Jen Easterly</t>
+          <t>Hafsa Amjad</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Cybersecurity and Infrastructure Security Agency CISA</t>
+          <t>AIM Academy Center</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Cybersecurity and Infrastructure Security Agency CISA</t>
+          <t>AIM Academy Center</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.aimacademycenter.com</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Anne Neuberger</t>
+          <t>Julia Autry</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>The White House</t>
+          <t>Brush Cyber</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Deputy National Security Advisor for Cyber and Emerging Technology</t>
+          <t>Cyber Defense Incident Responder</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>The White House</t>
+          <t>Brush Cyber</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://brushcyber.com</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Christopher Krebs</t>
+          <t>Swati Babbar</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Krebs Stamos Group</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Former Director of CISA &amp; Founding Partner</t>
+          <t>Application Security Engineer</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Krebs Stamos Group</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
+          <t>https://www.amazon.com</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.linkedin.com/in/swatibabbar</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Kemba Walden</t>
+          <t>Bill Bernard</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Office of the National Cyber Director</t>
+          <t>Between Two Firewalls</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Former Acting National Cyber Director</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Office of the National Cyber Director</t>
+          <t>Between Two Firewalls</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.betweentwofirewalls.com</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Chris Inglis</t>
+          <t>James Bierly</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>National Cyber Directorate Advisory Board</t>
+          <t>Secure Point Solutions</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Former US National Cyber Director &amp; Advisory Board Member</t>
+          <t>Co-Founder/Principal Security Consultant</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>National Cyber Directorate Advisory Board</t>
+          <t>Secure Point Solutions</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://securepointsolutions.com</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Rob Joyce</t>
+          <t>Michael Boddicker</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>National Security Agency NSA</t>
+          <t>City of Davenport</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Former Director of Cybersecurity</t>
+          <t>I.T. Director</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>National Security Agency NSA</t>
+          <t>City of Davenport</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.davenportiowa.com</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Eric Goldstein</t>
+          <t>Doug Brush</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Cybersecurity and Infrastructure Security Agency CISA</t>
+          <t>Brush Cyber</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Executive Assistant Director for Cybersecurity</t>
+          <t>Cyber Personal Trainer | Special Master</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Cybersecurity and Infrastructure Security Agency CISA</t>
+          <t>Brush Cyber</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
+          <t>https://brushcyber.com</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.linkedin.com/in/douglasabrush</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Brandon Wales</t>
+          <t>Brandon Colley</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Cybersecurity and Infrastructure Security Agency CISA</t>
+          <t>TrustedSec</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Former Executive Director</t>
+          <t>Senior Security Consultant</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Cybersecurity and Infrastructure Security Agency CISA</t>
+          <t>TrustedSec</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.trustedsec.com</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Bryan Vorndran</t>
+          <t>Joshua Corman</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Federal Bureau of Investigation FBI</t>
+          <t>Institute for Security and Technology (IST)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Assistant Director, Cyber Division</t>
+          <t>Executive in Residence</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Federal Bureau of Investigation FBI</t>
+          <t>Institute for Security and Technology (IST)</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
+          <t>https://securityandtechnology.org</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.linkedin.com/in/cormanjoshua</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Harry Coker Jr.</t>
+          <t>Joshua Crumbaugh</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>The White House</t>
+          <t>PhishFirewall, Inc</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>National Cyber Director</t>
+          <t>Founder/CEO</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>The White House</t>
+          <t>PhishFirewall, Inc</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://phishfirewall.com</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>David Cattler</t>
+          <t>John Aron</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Defense Counterintelligence and Security Agency DCSA</t>
+          <t>Aronetics</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Founder and CEO</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Defense Counterintelligence and Security Agency DCSA</t>
+          <t>Aronetics</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Quantico, VA, USA</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.aronetics.com</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Nathaniel Fick</t>
+          <t>Michael Daugherty</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>US Department of State</t>
+          <t>LabMD</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Ambassador at Large for Cyberspace and Digital Policy</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>US Department of State</t>
+          <t>LabMD</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
+          <t>https://www.labmd.com</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.linkedin.com/in/michael-j-daugherty-7a500819</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Kevin Mandia</t>
+          <t>Aj Debole</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Mandiant / Google Cloud</t>
+          <t>Oracle</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>Field Chief Information Security Officer (CISO)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Mandiant / Google Cloud</t>
+          <t>Oracle</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Reston, VA, USA</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.oracle.com</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Matthew Travis</t>
+          <t>Louis DeWeaver</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>US National Cyber &amp; Cloud Security Summit</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>The Cyber AB</t>
+          <t>Marsh McLennan Agency</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>Cyber Security Consultant</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>The Cyber AB</t>
+          <t>Marsh McLennan Agency</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on Secure by Design principles, Federal Cyber Defense Infrastructure, Zero Trust Architecture, ransomware task force operations, and national critical infrastructure protection (RSA Conference, Black Hat USA, DEF CON).</t>
+          <t>https://www.marshmclennanagency.com</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Jarrod Gingras</t>
+          <t>Arad Donenfeld</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Real Story Group</t>
+          <t>SafeBreach</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Managing Director &amp; DAM Analyst</t>
+          <t>Attacks and Exploits Developer</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Real Story Group</t>
+          <t>SafeBreach</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://safebreach.com</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Mike Szumlinski</t>
+          <t>Sean Donovan</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Backlight</t>
+          <t>Red Sky Consulting</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Field Chief Technology Officer</t>
+          <t>Founder &amp; CEO</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Backlight</t>
+          <t>Red Sky Consulting</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>https://redskyconsulting.com</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.linkedin.com/in/seandonovanredsky</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>John Horodyski</t>
+          <t>Shane Dwyer</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Salt Flats</t>
+          <t>State of Iowa</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Executive Director, Information &amp; Data Strategy</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Salt Flats</t>
+          <t>State of Iowa</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>https://iowa.gov</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.linkedin.com/in/shanedwyer</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Theresa Regli</t>
+          <t>JD Eger</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Independent Consultant</t>
+          <t>ThreatLocker</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Digital Asset Strategist &amp; Author</t>
+          <t>Solutions Engineer</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Independent Consultant</t>
+          <t>ThreatLocker</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Boston, MA, USA</t>
+          <t>https://www.threatlocker.com</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.linkedin.com/in/jdeger</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Graham Allan</t>
+          <t>David Etue</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>The Home Depot</t>
+          <t>Cyberbit</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Senior Manager, Content Architecture &amp; DAM</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>The Home Depot</t>
+          <t>Cyberbit</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Atlanta, GA, USA</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.cyberbit.com</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>David Lipsey</t>
+          <t>Gadi Evron</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>The DAM Foundation</t>
+          <t>Knostic</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Chair</t>
+          <t>CEO and Founder &amp; CISO-in-Residence at CSA</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>The DAM Foundation</t>
+          <t>Knostic</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Philadelphia, PA, USA</t>
+          <t>https://knostic.ai</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.linkedin.com/in/gadievron</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Cynthia Simpson</t>
+          <t>Bob Flores</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>The Estée Lauder Companies</t>
+          <t>Applicology Incorporated</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Global DAM &amp; Creative Operations Director</t>
+          <t>President &amp; CEO</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>The Estée Lauder Companies</t>
+          <t>Applicology Incorporated</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>https://www.applicology.com</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.linkedin.com/in/bob-flores-00216b2</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Frederic Sanuy</t>
+          <t>Laszlo Gonc</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Activo DAM Consulting</t>
+          <t>Next Era Transformation Group, LLC</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>CEO &amp; Chief Solutions Architect</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Activo DAM Consulting</t>
+          <t>Next Era Transformation Group, LLC</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.nexteraenergy.com</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Mark Davey</t>
+          <t>Paul Grabow</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>The CODIFY Group</t>
+          <t>Cybersecurity CMMC Advisors, LLC</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Founder &amp; Director</t>
+          <t>Principal Researcher/Advisor</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>The CODIFY Group</t>
+          <t>Cybersecurity CMMC Advisors, LLC</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>London / New York, USA</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.cybersecuritycmmcadvisorsllc.com</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Jennifer Allen</t>
+          <t>Richard Greenberg</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Sony Pictures Entertainment</t>
+          <t>Security Advisors LLC</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Director of Global Asset Management &amp; Content Systems</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Sony Pictures Entertainment</t>
+          <t>Security Advisors LLC</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, USA</t>
+          <t>https://www.securityadvisors.net</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.linkedin.com/in/richard-greenberg-063772144</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Linda Tadic</t>
+          <t>Sebastiaan Gybels</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Digital Bedrock</t>
+          <t>Northern Trust</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>CEO &amp; Founder</t>
+          <t>SVP Cyber Security</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Digital Bedrock</t>
+          <t>Northern Trust</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, USA</t>
+          <t>https://www.northerntrust.com</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.linkedin.com/in/sebastiaangybels</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Craig Llewellyn</t>
+          <t>Travis Hartman</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>MANTECH</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Director of Enterprise Creative Tech</t>
+          <t>Senior Technical Director</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>MANTECH</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.mantech.com</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Ian Matzen</t>
+          <t>Corey Hlavacek</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>NBCUniversal</t>
+          <t>enVista</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Metadata &amp; Taxonomy Lead</t>
+          <t>Senior Director Information Security</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>NBCUniversal</t>
+          <t>enVista</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.envistacorp.com</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Reem El Asaleh</t>
+          <t>Steve Hunt</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Toronto Metropolitan University</t>
+          <t>Impact Leaders</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Executive Advisor</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Toronto Metropolitan University</t>
+          <t>Impact Leaders</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Toronto / New York, USA</t>
+          <t>https://www.impactleaders.com</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.linkedin.com/in/stevehunt</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Erik Bernhardsson</t>
+          <t>Chris Johnson</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>GTIA</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Founder &amp; CEO</t>
+          <t>Director of Cybersecurity Programs and Executive Director of GTIA ISAO</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>GTIA</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>https://www.gtia.com</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Modal founder &amp; CEO; pioneer in serverless container runtimes, GPU virtualization, and distributed systems. Keynotes at PyData, Strange Loop, MLSys.</t>
+          <t>https://www.linkedin.com/in/chrisjohnson1337msp</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Will Reese</t>
+          <t>John Johnson</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Docent Institute</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Founding Engineer &amp; Systems Architect</t>
+          <t>Founder/President/Chairman</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Docent Institute</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>https://corncon.net</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Modal founding engineer specializing in microVM architecture, Linux cgroups, and high-throughput container virtualization.</t>
+          <t>https://www.linkedin.com/in/john-d-johnson-ph-d-cissp-9226191</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Akshat Bubna</t>
+          <t>Arjun Katneni</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>SolarWinds</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>AI Infrastructure Lead</t>
+          <t>Lead Security Engineer</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>SolarWinds</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Modal engineering lead for distributed GPU inference, model sharding, and cluster auto-scaling.</t>
+          <t>https://www.solarwinds.com</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Jonathon Belotti</t>
+          <t>Kristin King</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>AnzenSage</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Staff Systems Engineer</t>
+          <t>CEO &amp; Founder, Podcast Host &amp; Author</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>AnzenSage</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>https://anzensage.com</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Systems architect for distributed execution engines, low-latency microVM architecture, and edge runtimes.</t>
+          <t>https://www.linkedin.com/in/kingmkristin</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Charles Fry</t>
+          <t>Zach Kromkowski</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Senteon.io</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Distributed Systems Lead</t>
+          <t>CRO</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Modal Labs</t>
+          <t>Senteon.io</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Cloud infrastructure architect; speaker on large-scale cluster orchestration and resilient workload scheduling.</t>
+          <t>https://www.senteonio.com</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Luis Ceze</t>
+          <t>Kate Kuehn</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>University of Washington &amp; OctoAI</t>
+          <t>WWT</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>CEO &amp; Professor of Computer Science</t>
+          <t>Global Head of Cyber Advocacy</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>University of Washington &amp; OctoAI</t>
+          <t>WWT</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Seattle, WA, USA</t>
+          <t>https://www.wwt.com</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>UW Professor &amp; OctoAI CEO; keynote speaker at ASPLOS, ISCA, NeurIPS on hardware-software co-design for AI and efficient deep learning compilation.</t>
+          <t>https://www.linkedin.com/in/katekuehn</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Tri Dao</t>
+          <t>Bobby Kuzma</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Together AI &amp; Princeton University</t>
+          <t>Marqui Security</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Chief Scientist &amp; Assistant Professor</t>
+          <t>Director of Cyber Threat Intelligence / CISO</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Together AI &amp; Princeton University</t>
+          <t>Marqui Security</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Princeton, NJ, USA</t>
+          <t>https://www.marquisecurity.com</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Creator of FlashAttention; invited speaker at NeurIPS, ICML, MLSys on linear and sub-quadratic attention architectures and kernel optimization.</t>
+          <t>https://www.linkedin.com/in/bobbykuzma</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Horace He</t>
+          <t>John Kwarsick</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>PyTorch Core &amp; Meta AI</t>
+          <t>Kwarsick Consulting, LLC</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Machine Learning Systems Engineer</t>
+          <t>Founder and Principal Consultant</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>PyTorch Core &amp; Meta AI</t>
+          <t>Kwarsick Consulting, LLC</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>PyTorch core engineer; speaker on torch.compile, compiler optimizations, GPU kernel codegen, and tensor program synthesis.</t>
+          <t>https://www.kwarsickconsultingllc.com</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Tim Dettmers</t>
+          <t>Fred Kwong</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Allen Institute for AI &amp; University of Washington</t>
+          <t>DeVry University</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Assistant Professor &amp; Research Scientist</t>
+          <t>VP, Chief Information Security Officer</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Allen Institute for AI &amp; University of Washington</t>
+          <t>DeVry University</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Seattle, WA, USA</t>
+          <t>https://www.devry.edu</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Creator of bitsandbytes (8-bit &amp; 4-bit quantization, QLoRA); keynote speaker on efficient deep learning and memory-bounded LLM fine-tuning.</t>
+          <t>https://www.linkedin.com/in/fredkwong</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Bert Maher</t>
+          <t>Naveen Konrajankuppam Mahavishnu</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Meta AI</t>
+          <t>Aira Security</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Compiler Engineering Lead</t>
+          <t>CTO</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Meta AI</t>
+          <t>Aira Security</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Menlo Park, CA, USA</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Meta AI compiler lead; technical talks on deep learning compilers, AOTInductor, and high-performance ML inference backends.</t>
+          <t>https://www.airasecurity.com</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Dan Fu</t>
+          <t>Jeff Man</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Stanford University &amp; Cartesia</t>
+          <t>Secure Ideas, LLC</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>AI Systems Researcher</t>
+          <t>Executive Director - PCI</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Stanford University &amp; Cartesia</t>
+          <t>Secure Ideas, LLC</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Stanford, CA, USA</t>
+          <t>https://www.secureideas.com</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Co-creator of FlashAttention, H3, and Monarch architectures; speaker on efficient long-context sequence modeling at ICML and MLSys.</t>
+          <t>https://www.linkedin.com/in/jeff-man-pci</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Sarah Catanzaro</t>
+          <t>Mitchell Marasch</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Amplify Partners</t>
+          <t>OnDefend</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>General Partner</t>
+          <t>Senior Red Team Penetration Tester</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Amplify Partners</t>
+          <t>OnDefend</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>Keynote speaker on AI infrastructure investing, open-source AI ecosystems, and developer tooling at Scale AI and O'Reilly Strata.</t>
+          <t>https://www.ondefend.com</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Beidi Chen</t>
+          <t>Richard H. L. Marshall</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Carnegie Mellon University</t>
+          <t>CinturionGroup</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Founder and Chairman of the Board</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Carnegie Mellon University</t>
+          <t>CinturionGroup</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, USA</t>
+          <t>https://www.cinturiongroup.com</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>CMU faculty; invited speaker on algorithm-hardware co-design for efficient LLM training and inference at MLSys and CVPR.</t>
+          <t>https://www.linkedin.com/in/richard-marshall-246008429</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Greg Brockman</t>
+          <t>Dwayne McDaniel</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Runtime by Modal</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>GitGuardian</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>President &amp; Co-Founder</t>
+          <t>Principal Developer Advocate</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>GitGuardian</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>https://www.gitguardian.com</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>OpenAI President &amp; Co-founder; keynote addresses at SXSW, TechCrunch Disrupt, and MIT on scaling laws, supercomputing infrastructure, and frontier AI models.</t>
+          <t>https://www.linkedin.com/in/dwaynemcdaniel</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Sandra Hundacker</t>
+          <t>Richard Noel</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Rick Steves' Europe</t>
+          <t>Eptura</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Creative &amp; Operations Director</t>
+          <t>Director, Security Operations and Infrastructure</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Rick Steves' Europe</t>
+          <t>Eptura</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Edmonds, WA, USA</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://eptura.com</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Orin Dubrow</t>
+          <t>Kasi Paturi</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>DAM New York 2026</t>
+          <t>CornCon Cybersecurity Conference</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Rick Steves' Europe</t>
+          <t>Pan Asian American Business Council</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Creative Operations &amp; Production Specialist</t>
+          <t>President</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Rick Steves' Europe</t>
+          <t>Pan Asian American Business Council</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Edmonds, WA, USA</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Keynotes on AI and Metadata Automation in Global Asset Supply Chains at Henry Stewart DAM Europe, Creative Operations Exchange, and International DAM Symposium.</t>
+          <t>https://www.panasianamericanbusinesscouncil.com</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Jacob Pender</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Black Hawk College</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Black Hawk College</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bhc.edu</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Tuan Phan</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>ThreatReel</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>AVP | Data Security and Insider Threat Strategy</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>ThreatReel</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>https://threatreel.com</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Bruce Phillips</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Williston Financial Group (WFG)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>SVP &amp; Chief Information Security Officer</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Williston Financial Group (WFG)</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>https://wfgtitle.com</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/brucephillips</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Ken Reaves</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Relate Central</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Relate Central</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.relatecentral.com</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kenreaves</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Paul Rice</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>PayPal Inc</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Sr. Counsel, Cybersecurity-Legal</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>PayPal Inc</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.paypal.com</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Launa Rich</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>QuickStart</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Cyber Skills &amp; Talent Intelligence Leader</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>QuickStart</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.quickstart.com</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr"/>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Randy Rose</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Center for Internet Security</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>VP, Security Operations &amp; Intelligence</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Center for Internet Security</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cisecurity.org</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/randy-rose-94b85234</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Jason Rowland</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Evolve Security</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Chief Delivery Officer</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Evolve Security</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.evolvesecurity.com</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jasonrrowland</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Richard Rushing</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Motorola Mobility</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>CISO</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Motorola Mobility</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.motorola.com</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/richardrushing</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Greg Schaffer</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>vCISO Services, LLC</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>vCISO Services, LLC</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.vcisoservicesllc.com</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/gregschaffer</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Matt Scheurer</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>First Financial Bank</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>VP, Computer Security &amp; Incident Response</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>First Financial Bank</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bankatfirst.com</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/scubamatt</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Winn Schwartau</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive Security Institute</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Director of Special Projects</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive Security Institute</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>https://cognitivesecurityinstitute.org</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/winnschwartau</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Mayank Sethi</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Group1001</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Principal Data Operations Engineer</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Group1001</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.group1001.com</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sethi-m</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Steve Shelton</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Green Shoe</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Founder &amp; Chief Resilience Officer</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Green Shoe</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.greenshoe.com</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr"/>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Carl Shimel</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Obsidian Security</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Head of Threat Intelligence</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Obsidian Security</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>https://www.obsidiansecurity.com</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr"/>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Ken Smith</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>CyberproAI</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Director of Solutions and Strategic Partnerships</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>CyberproAI</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>https://cyberproai.com</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/signalsec</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Nidhi Srivastava</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>DigiArmorX LLC</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>DigiArmorX LLC</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>https://www.digiarmorxllc.com</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr"/>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Aaileen Sarwar Syed</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Girls Who Code</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Girls Who Code</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>https://girlswhocode.com</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr"/>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Paula Januszkiewicz</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>CQURE</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>CQURE</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>https://cqure.net</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/paulajanuszkiewicz</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Jayson E. Street</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Illicit Strategies</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Chief Adversarial Strategies</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Illicit Strategies</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>https://illicitstrategies.com</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jaysonestreet</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Ira Winkler</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>CYE</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Field CISO &amp; Vice President</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>CYE</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>https://cyesec.com</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/irawinkler</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Chloe Messdaghi</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Head of Threat Intelligence</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>https://block.xyz</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/chloemessdaghi</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Gene Spafford</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>CERIAS Purdue University</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Executive Director Emeritus</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>CERIAS Purdue University</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cerias.purdue.edu</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/spaf</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Joseph Purita</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>AASCP Fall Regenerative Medicine Conference Miami 2026</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>The Institute of Regenerative Medicine</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Chief Medical Officer</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>The Institute of Regenerative Medicine</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>https://stemcellrevolution.com</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/joe-purita-9b8695118</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>USA, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Peter Verlander</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>AASCP Fall Regenerative Medicine Conference Miami 2026</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>BioXcel Therapeutics</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Vice President of Research &amp; Development</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>BioXcel Therapeutics</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bioxceltherapeutics.com</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/peter-verlander-phd</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>USA, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Douglas Spiel</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>AASCP Fall Regenerative Medicine Conference Miami 2026</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Spiel MD</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Founder &amp; Radiologist</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Spiel MD</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.spielmd.com</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/douglas-spiel-11b52b25</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>USA, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Sheldon Jordan</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>AASCP Fall Regenerative Medicine Conference Miami 2026</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>The Regenesis Project</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Neurologist &amp; Director</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>The Regenesis Project</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>https://www.theregenesisproject.com</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr"/>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>USA, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Alimorad Farshchian</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>AASCP Fall Regenerative Medicine Conference Miami 2026</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>The Center for Regenerative Medicine</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Medical Director &amp; Founder</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>The Center for Regenerative Medicine</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thecenterforregenerativemedicine.com</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr"/>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>USA, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Charles Runels</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>AASCP Fall Regenerative Medicine Conference Miami 2026</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Cellular Medicine Association</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Clinical Researcher &amp; Founder</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Cellular Medicine Association</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cellularmedicineassociation.com</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/charles-runels-md-80633211</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>USA, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Sharon McQuillan</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>AASCP Fall Regenerative Medicine Conference Miami 2026</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Ageless Regenerative Institute</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Founder &amp; Medical Director</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Ageless Regenerative Institute</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.agelessregenerativeinstitute.com</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/doctormcquillan</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>USA, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Susan Kressly</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>American Academy of Pediatrics</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>American Academy of Pediatrics</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aap.org</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/susan-kressly-md</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>Washington, DC, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Mark Del Monte</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>American Academy of Pediatrics</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>CEO &amp; Executive Vice President</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>American Academy of Pediatrics</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aap.org</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mark-del-monte-380b8b9</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Washington, DC, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Sandy Chung</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>American Academy of Pediatrics</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Immediate Past President</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>American Academy of Pediatrics</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aap.org</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sandychung</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>Washington, DC, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Megan Holliday</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>IOActive, Inc</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Security Consultant</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>IOActive, Inc</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>https://ioactive.com</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/megan-holliday</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Rob Labbe</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Mm-ISAC</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>CISO in Residence</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Mm-ISAC</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mmisac.com</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rob-labbe</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Corey Munson</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>PC Matic</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Vice President</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>PC Matic</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pcmatic.com</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/corey-munson</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Niharika P Pujari</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>McGraw Hill</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Lead Software Engineer</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>McGraw Hill</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mheducation.com</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/niharika-p-pujari</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Michael Ratemo</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Cyber Security Simplified</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Principal Security Advisor</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Cyber Security Simplified</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cybersecuritysimplified.com</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michael-ratemo</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Tanya Janca</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>We Hack Purple</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>We Hack Purple</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>https://wehackpurple.com</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tanya-janca</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Tackett</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Secure Ideas</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Secure Ideas</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.secureideas.com</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kevintackett</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Cyrus Walker</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Data Defenders</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Founder, CEO</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Data Defenders</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>https://www.datadefenders.com</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/cyruswalker</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Rakshan Urooj Syed</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Lewis University</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Lewis University</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.lewisu.edu</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr"/>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>Derrick Thomas</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Solution Manager II / Deputy Cyber Operations Lead at Deloitte</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>https://www.deloitte.com</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/derrickthomas1</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Jaime Urteaga</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>HealthTech</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>GRC Leader</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>HealthTech</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>https://www.healthtech.com</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr"/>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Mohankumar Vengatachalam</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Aira Security</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Aira Security</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>https://www.airasecurity.com</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr"/>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Robert Wagner</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>ISSA Chicago</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Advisory CISO</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>ISSA Chicago</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>https://www.issachicago.com</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/robert-wagner-ciso</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Aakash Abhay Yadav</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Cerebras</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Cybersecurity GRC Manager| OWASP AI Exchange Author</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Cerebras</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cerebras.ai</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr"/>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Lintile</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>DFIU.tv</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Game Show Host</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>DFIU.tv</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dfiu.tv</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr"/>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Dave Lewis</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>CornCon Cybersecurity Conference</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Cisco</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Global Advisory CISO</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Cisco</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cisco.com</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/gattaca</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>Davenport, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>Benjamin Hoffman</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Oregon Health &amp; Science University (OHSU)</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Professor of Pediatrics &amp; Chair of Injury Prevention</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Oregon Health &amp; Science University (OHSU)</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ohsu.edu</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/benjamin-hoffman-md</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>Washington, DC, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Moira Szilagyi</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>UCLA Mattel Children's Hospital</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Professor of Pediatrics</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>UCLA Mattel Children's Hospital</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>https://www.uclahealth.org/mattel</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/moira-szilagyi-md-phd</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>Washington, DC, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>Lee Savio Beers</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Children's National Hospital</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Past President &amp; Medical Director</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Children's National Hospital</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>https://childrensnational.org</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/lee-savio-beers-md</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>Washington, DC, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>Colleen Kraft</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Keck School of Medicine of USC</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Clinical Professor of Pediatrics</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Keck School of Medicine of USC</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>https://keck.usc.edu</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/colleen-kraft-24037736</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>Washington, DC, USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Yasuda</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>AAP National Conference &amp; Exhibition 2026</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>University of Washington School of Medicine</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>Clinical Professor Emeritus</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>University of Washington School of Medicine</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>https://www.washington.edu</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kyle-yasuda-md</t>
+        </is>
+      </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>Seattle, WA, USA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adding a scraping sources
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -464,10 +464,10 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="33" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
     <col width="109" customWidth="1" min="11" max="11"/>
     <col width="109" customWidth="1" min="12" max="12"/>
     <col width="109" customWidth="1" min="13" max="13"/>
@@ -621,17 +621,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>CONF-2026-E8124C</t>
+          <t>CONF-2026-31CDFC</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>CONGRESO 7 HORAS EN SU PRESENCIA (OCTUBRE 8 AL 11, 2026)</t>
+          <t>New York Comic Con - 4 Day Pass</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Religion &amp; Spirituality</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -651,12 +651,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Hyvee Arena</t>
+          <t>Jacob Javits Center, USA</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -666,39 +666,39 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>PASTOR JUAN CARLOS HARRIGAN</t>
+          <t>Allevents Conference Network</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/congreso-7-horas-en-su-presencia-octubre-8-al-11-2026-tickets-1983897931117</t>
+          <t>https://allevents.in/new-york/new-york-comic-con-4-day-pass/210002445807870</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/congreso-7-horas-en-su-presencia-octubre-8-al-11-2026-tickets-1983897931117</t>
+          <t>https://allevents.in/new-york/new-york-comic-con-4-day-pass/210002445807870</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/congreso-7-horas-en-su-presencia-octubre-8-al-11-2026-tickets-1983897931117</t>
+          <t>https://allevents.in/new-york/new-york-comic-con-4-day-pass/210002445807870</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CONF-2026-89AD50</t>
+          <t>CONF-2026-D40151</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
+          <t>Surviving the 2:00 AM Automated Job Rejection: NYC</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -718,13 +718,17 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>555 Broadway, USA</t>
+        </is>
+      </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -734,22 +738,22 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Luma Tech Discovery</t>
+          <t>Allevents Conference Network</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>https://lu.ma/gbdkbar8</t>
+          <t>https://allevents.in/new-york/surviving-the-2-00-am-automated-job-rejection-nyc-tickets/80002710348001</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>https://lu.ma/gbdkbar8</t>
+          <t>https://allevents.in/new-york/surviving-the-2-00-am-automated-job-rejection-nyc-tickets/80002710348001</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>https://lu.ma/gbdkbar8</t>
+          <t>https://allevents.in/new-york/surviving-the-2-00-am-automated-job-rejection-nyc-tickets/80002710348001</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -761,12 +765,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>CONF-2026-902EE8</t>
+          <t>CONF-2026-89AD50</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -786,19 +790,15 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>USA</t>
@@ -811,17 +811,17 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://lu.ma/gbdkbar8</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://lu.ma/gbdkbar8</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://lu.ma/gbdkbar8</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
@@ -833,17 +833,17 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>CONF-2026-C93491</t>
+          <t>CONF-2026-902EE8</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Holy Spirit Encounter Services - Phoenix, AZ</t>
+          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Religion &amp; Spirituality</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -863,12 +863,12 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>9620 N Metro Pkwy W ste 135</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -878,99 +878,243 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>David Hernandez Ministries</t>
+          <t>Luma Tech Discovery</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/holy-spirit-encounter-services-phoenix-az-october-8-9th-tickets-1992584947216</t>
+          <t>https://lu.ma/lnnlfa87</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/holy-spirit-encounter-services-phoenix-az-october-8-9th-tickets-1992584947216</t>
+          <t>https://lu.ma/lnnlfa87</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/holy-spirit-encounter-services-phoenix-az-october-8-9th-tickets-1992584947216</t>
+          <t>https://lu.ma/lnnlfa87</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>CONF-2026-C93491</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Holy Spirit Encounter Services - Phoenix, AZ</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Religion &amp; Spirituality</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>9620 N Metro Pkwy W ste 135</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Phoenix</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>David Hernandez Ministries</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/holy-spirit-encounter-services-phoenix-az-october-8-9th-tickets-1992584947216</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/holy-spirit-encounter-services-phoenix-az-october-8-9th-tickets-1992584947216</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/holy-spirit-encounter-services-phoenix-az-october-8-9th-tickets-1992584947216</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>CONF-2026-DAF985</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Legacy Conference 2026</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Religion &amp; Spirituality</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>2026-10-10</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Nashville Municipal Auditorium</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Nashville</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>Legacy Nashville</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Legacy Nashville</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/legacy-conference-2026-oct-8-10-tickets-1787167759879</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/legacy-conference-2026-oct-8-10-tickets-1787167759879</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/legacy-conference-2026-oct-8-10-tickets-1787167759879</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CONF-2026-132239</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>PaleyFest NY 2026: American Horror Story - 13</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Paley Center For Media, New York, NY, USA</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Allevents Conference Network</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/paleyfest-ny-2026-american-horror-story-13/2300030592329659</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/paleyfest-ny-2026-american-horror-story-13/2300030592329659</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/paleyfest-ny-2026-american-horror-story-13/2300030592329659</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adding a email feature and testing
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -559,17 +559,17 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-7933B9</t>
+          <t>CONF-2026-6E93C3</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Open Source AI Stack: Models, Inference, and Agent Harness</t>
+          <t>Claude Build Day | Mental Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>AI Solutions</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -604,22 +604,22 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>Luma Tech Discovery</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/novita-oas6</t>
+          <t>https://lu.ma/claude-r5w5</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/novita-oas6</t>
+          <t>https://lu.ma/claude-r5w5</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/novita-oas6</t>
+          <t>https://lu.ma/claude-r5w5</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
@@ -631,12 +631,12 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-4BC11E</t>
+          <t>CONF-2026-7933B9</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Building at the Frontier: Hypergrowth Startup Operator Panel</t>
+          <t>Open Source AI Stack: Models, Inference, and Agent Harness</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -681,17 +681,17 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/m2o3zerh</t>
+          <t>https://lu.ma/novita-oas6</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/m2o3zerh</t>
+          <t>https://lu.ma/novita-oas6</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/m2o3zerh</t>
+          <t>https://lu.ma/novita-oas6</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
@@ -703,17 +703,17 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-6E93C3</t>
+          <t>CONF-2026-4BC11E</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>Building at the Frontier: Hypergrowth Startup Operator Panel</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>AI Solutions</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -748,22 +748,22 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Luma Tech Discovery</t>
+          <t>Luma Conference Network</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/claude-r5w5</t>
+          <t>https://lu.ma/m2o3zerh</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/claude-r5w5</t>
+          <t>https://lu.ma/m2o3zerh</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/claude-r5w5</t>
+          <t>https://lu.ma/m2o3zerh</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
@@ -775,12 +775,12 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-3B6843</t>
+          <t>CONF-2026-902EE8</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
+          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -820,22 +820,22 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>Luma Tech Discovery</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/gbdkbar8</t>
+          <t>https://lu.ma/lnnlfa87</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/gbdkbar8</t>
+          <t>https://lu.ma/lnnlfa87</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/gbdkbar8</t>
+          <t>https://lu.ma/lnnlfa87</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -847,12 +847,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-902EE8</t>
+          <t>CONF-2026-3B6843</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -877,14 +877,14 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
+          <t>San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
           <t>USA</t>
@@ -892,22 +892,22 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Luma Tech Discovery</t>
+          <t>Luma Conference Network</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://lu.ma/gbdkbar8</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://lu.ma/gbdkbar8</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://lu.ma/gbdkbar8</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
@@ -933,9 +933,9 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="86" customWidth="1" min="3" max="3"/>
-    <col width="73" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="4" max="4"/>
     <col width="86" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
     <col width="53" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
@@ -985,7 +985,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Amy Lin</t>
+          <t>Keith Peiris</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -995,49 +995,49 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>Lightfield</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Event Host &amp;</t>
+          <t>CEO and Co-founder</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>Lightfield</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>https://www.lumaconferencenetwork.com</t>
+          <t>https://lightfield.app</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/heyamylin</t>
+          <t>https://www.linkedin.com/in/keithpeiris</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, USA</t>
+          <t>San Francisco, CA, USA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Keith Peiris</t>
+          <t>Jeffrey Morgan</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
+          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Lightfield</t>
+          <t>Ollama</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -1047,17 +1047,17 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Lightfield</t>
+          <t>Ollama</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>https://lightfield.app</t>
+          <t>https://ollama.com</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/keithpeiris</t>
+          <t>https://www.linkedin.com/in/jmorganca</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Jeffrey Morgan</t>
+          <t>Michael Elabd</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1079,27 +1079,27 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Ollama</t>
+          <t>Trajectory</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>CEO and Co-founder</t>
+          <t>Co-founder</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Ollama</t>
+          <t>Trajectory</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>https://ollama.com</t>
+          <t>https://trajectory.ai</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jmorganca</t>
+          <t>https://www.linkedin.com/in/michael-elabd</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -1111,7 +1111,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Michael Elabd</t>
+          <t>Erwan Menard</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1121,27 +1121,27 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Trajectory</t>
+          <t>Crusoe</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Co-founder</t>
+          <t>SVP of Product Management</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Trajectory</t>
+          <t>Crusoe</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>https://trajectory.ai</t>
+          <t>https://crusoe.ai</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/michael-elabd</t>
+          <t>https://www.linkedin.com/in/erwanmenard</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1153,91 +1153,91 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Erwan Menard</t>
+          <t>Sharon Rao</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>Claude Build Day | Mental Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Crusoe</t>
+          <t>medschoolbro</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>SVP of Product Management</t>
+          <t>- Former MD / 1x Founder / Ex-COO</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Crusoe</t>
+          <t>medschoolbro</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>https://crusoe.ai</t>
+          <t>https://www.medschoolbro.com</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/erwanmenard</t>
+          <t>https://www.linkedin.com/in/sharonrao</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, USA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Judy Wu</t>
+          <t>Brandon Slicklein</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>Claude Build Day | Mental Health &amp; Wellness</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>AuraPath AI. I build AI-native products for clients and teach others to do the same</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Event Host &amp;</t>
+          <t>Co-founder</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>AuraPath AI. I build AI-native products for clients and teach others to do the same</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>https://www.lumaconferencenetwork.com</t>
+          <t>https://aurapath.ai</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/wujudy</t>
+          <t>https://www.linkedin.com/in/brandon-slicklein</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Prasanna Gopalakrishnan</t>
+          <t>Abhay Garg</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1247,27 +1247,27 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>MotionSyncHealth</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Chief AI officer and Chief product officer. Board Director | LinkedIn:</t>
+          <t>Founding Engineer | HealthTech AI | Co-Founder</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>MotionSyncHealth</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>https://www.lumaconferencenetwork.com</t>
+          <t>https://motionsynchealth.com</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/prasannagopalakrishnan</t>
+          <t>https://www.linkedin.com/in/gargabhay06</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1279,91 +1279,91 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Sharon Rao</t>
+          <t>Amy Lin</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>medschoolbro</t>
+          <t>Outcast Ventures</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>- Former MD / 1x Founder / Ex-COO</t>
+          <t>Partner &amp; Event Host</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>medschoolbro</t>
+          <t>Outcast Ventures</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>https://www.medschoolbro.com</t>
+          <t>https://outcast.vc</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sharonrao</t>
+          <t>https://www.linkedin.com/in/heyamylin</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>New York, USA</t>
+          <t>San Francisco, USA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Brandon Slicklein</t>
+          <t>Judy Wu</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>AuraPath AI. I build AI-native products for clients and teach others to do the same</t>
+          <t>Luma</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Co-founder</t>
+          <t>Event Host &amp; Organizer</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>AuraPath AI. I build AI-native products for clients and teach others to do the same</t>
+          <t>Luma</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>https://aurapath.ai</t>
+          <t>https://lu.ma</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/brandon-slicklein</t>
+          <t>https://www.linkedin.com/in/wujudy</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>San Francisco, USA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Abhay Garg</t>
+          <t>Prasanna Gopalakrishnan</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1373,27 +1373,27 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>MotionSyncHealth</t>
+          <t>Enterprise AI</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Founding Engineer | HealthTech AI | Co-Founder</t>
+          <t>Chief AI Officer &amp; Board Director</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>MotionSyncHealth</t>
+          <t>Enterprise AI</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>https://motionsynchealth.com</t>
+          <t>https://lu.ma/claude-r5w5</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/gargabhay06</t>
+          <t>https://www.linkedin.com/in/prasannagopalakrishnan</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>MyWhatIf Foundation</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1425,12 +1425,12 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>MyWhatIf Foundation</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>https://www.lumaconferencenetwork.com</t>
+          <t>https://mywhatif.org</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>Luma</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1467,12 +1467,12 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>Luma</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>https://www.lumaconferencenetwork.com</t>
+          <t>https://lu.ma</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>Luma</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1509,12 +1509,12 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>Luma</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>https://www.lumaconferencenetwork.com</t>
+          <t>https://lu.ma</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
today conference details fetch
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -465,22 +465,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="67" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="47" customWidth="1" min="10" max="10"/>
+    <col width="73" customWidth="1" min="11" max="11"/>
+    <col width="73" customWidth="1" min="12" max="12"/>
+    <col width="76" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -559,27 +559,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-6E93C3</t>
+          <t>CONF-2026-SEALC1</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>2026 Seattle Lung Cancer Conference</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Medicine &amp; Hospitals</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Bell Harbor International Conference Center, 2211 Alaskan Way</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -604,54 +604,54 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Luma Tech Discovery</t>
+          <t>Binaytara Foundation</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/claude-r5w5</t>
+          <t>https://binaytara.org/conferences/seattle-lung-cancer-conference-2026/</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/claude-r5w5</t>
+          <t>https://binaytara.org/conferences/seattle-lung-cancer-conference-2026/</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/claude-r5w5</t>
+          <t>https://binaytara.org/conferences/seattle-lung-cancer-conference-2026/</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-7933B9</t>
+          <t>CONF-2026-AAO001</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Open Source AI Stack: Models, Inference, and Agent Harness</t>
+          <t>American Academy of Ophthalmology (AAO) 2026 Annual Meeting</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>AI Solutions</t>
+          <t>Medicine &amp; Hospitals</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Ernest N. Morial Convention Center, 900 Convention Center Blvd</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -676,54 +676,54 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>American Academy of Ophthalmology (AAO)</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/novita-oas6</t>
+          <t>https://www.aao.org/annual-meeting</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/novita-oas6</t>
+          <t>https://www.aao.org/annual-meeting/registration</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/novita-oas6</t>
+          <t>https://10times.com/aao-annual-meeting</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-4BC11E</t>
+          <t>CONF-2026-SKCOL1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Building at the Frontier: Hypergrowth Startup Operator Panel</t>
+          <t>Skin of Color Update 2026</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>AI Solutions</t>
+          <t>Medicine &amp; Hospitals</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>New York Hilton Midtown, 1335 Avenue of the Americas</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -748,54 +748,54 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Luma Conference Network</t>
+          <t>SanovaWorks / Skin of Color Society</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/m2o3zerh</t>
+          <t>https://skinofcolorupdate.com/</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/m2o3zerh</t>
+          <t>https://skinofcolorupdate.com/registration/</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/m2o3zerh</t>
+          <t>https://10times.com/skin-of-color-update</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-902EE8</t>
+          <t>CONF-2026-AMP001</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>Association of Medicine and Psychiatry (AMP) Annual Meeting 2026</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>AI Solutions</t>
+          <t>Healthcare / Medicine &amp; Hospitals</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -805,12 +805,12 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Hyatt Regency Newport Beach, 1107 Jamboree Rd</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New Newport Beach</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -820,99 +820,27 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Luma Tech Discovery</t>
+          <t>Association of Medicine and Psychiatry (AMP)</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://assocmedpsych.org/</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://assocmedpsych.org/annual-meeting</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://10times.com/association-of-medicine-and-psychiatry-annual-meeting</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CONF-2026-3B6843</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>AI Solutions</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, CA, USA</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Luma Conference Network</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>https://lu.ma/gbdkbar8</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>https://lu.ma/gbdkbar8</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>https://lu.ma/gbdkbar8</t>
-        </is>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
+          <t>2026-07-01</t>
         </is>
       </c>
     </row>
@@ -927,17 +855,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="86" customWidth="1" min="3" max="3"/>
-    <col width="49" customWidth="1" min="4" max="4"/>
-    <col width="86" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
-    <col width="53" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="67" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="67" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="51" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -985,542 +913,714 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Keith Peiris</t>
+          <t>Dr. Sid Devarakonda</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
+          <t>2026 Seattle Lung Cancer Conference</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Lightfield</t>
+          <t>Fred Hutchinson Cancer Center</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>CEO and Co-founder</t>
+          <t>Conference Co-Chair &amp; Associate Professor of Oncology</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Lightfield</t>
+          <t>Fred Hutchinson Cancer Center</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>https://lightfield.app</t>
+          <t>https://www.fredhutch.org</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/keithpeiris</t>
+          <t>https://www.linkedin.com/in/siddevarakonda</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Jeffrey Morgan</t>
+          <t>Dr. Lei Deng</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>2026 Seattle Lung Cancer Conference</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Ollama</t>
+          <t>Fred Hutchinson Cancer Center / UW Medicine</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>CEO and Co-founder</t>
+          <t>Conference Co-Chair &amp; Radiation Oncologist</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Ollama</t>
+          <t>UW Medicine</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>https://ollama.com</t>
+          <t>https://www.uwmedicine.org</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jmorganca</t>
+          <t>https://www.linkedin.com/in/lei-deng-md</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Michael Elabd</t>
+          <t>Dr. Matthew Gumbleton</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>2026 Seattle Lung Cancer Conference</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Trajectory</t>
+          <t>Huntsman Cancer Institute</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Co-founder</t>
+          <t>Thoracic Medical Oncologist &amp; Assistant Professor</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Trajectory</t>
+          <t>Huntsman Cancer Institute</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>https://trajectory.ai</t>
+          <t>https://healthcare.utah.edu/huntsmancancerinstitute</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/michael-elabd</t>
+          <t>https://www.linkedin.com/in/matthew-gumbleton</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Salt Lake City, UT</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Erwan Menard</t>
+          <t>Dr. Jeffrey P. Ward</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>2026 Seattle Lung Cancer Conference</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Crusoe</t>
+          <t>Washington University School of Medicine</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>SVP of Product Management</t>
+          <t>Associate Professor of Medicine &amp; Clinical Oncologist</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Crusoe</t>
+          <t>Washington University in St. Louis</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>https://crusoe.ai</t>
+          <t>https://wustl.edu</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/erwanmenard</t>
+          <t>https://www.linkedin.com/in/jeffrey-ward-md</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>St. Louis, MO</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Sharon Rao</t>
+          <t>Dr. Frank Weinberg</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>2026 Seattle Lung Cancer Conference</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>medschoolbro</t>
+          <t>University of Illinois Cancer Center</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>- Former MD / 1x Founder / Ex-COO</t>
+          <t>Assistant Professor of Medicine</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>medschoolbro</t>
+          <t>UI Cancer Center</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>https://www.medschoolbro.com</t>
+          <t>https://cancer.uillinois.edu</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sharonrao</t>
+          <t>https://www.linkedin.com/in/frank-weinberg</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>New York, USA</t>
+          <t>Chicago, IL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Brandon Slicklein</t>
+          <t>Dr. Jing Zeng</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>2026 Seattle Lung Cancer Conference</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>AuraPath AI. I build AI-native products for clients and teach others to do the same</t>
+          <t>University of Washington</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Co-founder</t>
+          <t>Professor of Radiation Oncology</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>AuraPath AI. I build AI-native products for clients and teach others to do the same</t>
+          <t>University of Washington</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>https://aurapath.ai</t>
+          <t>https://www.washington.edu</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/brandon-slicklein</t>
+          <t>https://www.linkedin.com/in/jing-zeng-md</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>New York, NY, USA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Abhay Garg</t>
+          <t>Dr. Stephen D. McLeod</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>American Academy of Ophthalmology (AAO) 2026 Annual Meeting</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>MotionSyncHealth</t>
+          <t>American Academy of Ophthalmology</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Founding Engineer | HealthTech AI | Co-Founder</t>
+          <t>Chief Executive Officer &amp; Clinical Professor</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>MotionSyncHealth</t>
+          <t>American Academy of Ophthalmology</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>https://motionsynchealth.com</t>
+          <t>https://www.aao.org</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/gargabhay06</t>
+          <t>https://www.linkedin.com/in/stephen-mcleod-aao</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>New York, USA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Amy Lin</t>
+          <t>Dr. Jane C. Edmond</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
+          <t>American Academy of Ophthalmology (AAO) 2026 Annual Meeting</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Outcast Ventures</t>
+          <t>Dell Medical School at UT Austin</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Partner &amp; Event Host</t>
+          <t>AAO Past President &amp; Department Chair of Ophthalmology</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Outcast Ventures</t>
+          <t>Dell Medical School</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>https://outcast.vc</t>
+          <t>https://dellmed.utexas.edu</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/heyamylin</t>
+          <t>https://www.linkedin.com/in/jane-edmond-md</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, USA</t>
+          <t>Austin, TX</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Judy Wu</t>
+          <t>Dr. Maria M. Aaron</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
+          <t>American Academy of Ophthalmology (AAO) 2026 Annual Meeting</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Luma</t>
+          <t>Emory Eye Center</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Event Host &amp; Organizer</t>
+          <t>Associate Dean of Graduate Medical Education &amp; Professor</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Luma</t>
+          <t>Emory University</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma</t>
+          <t>https://eyecenter.emory.edu</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/wujudy</t>
+          <t>https://www.linkedin.com/in/maria-aaron-md</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, USA</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Prasanna Gopalakrishnan</t>
+          <t>Dr. David W. Parke II</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>American Academy of Ophthalmology (AAO) 2026 Annual Meeting</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AI</t>
+          <t>American Academy of Ophthalmology</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Chief AI Officer &amp; Board Director</t>
+          <t>Executive Director &amp; Professor Emeritus</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AI</t>
+          <t>AAO</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/claude-r5w5</t>
+          <t>https://www.aao.org</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/prasannagopalakrishnan</t>
+          <t>https://www.linkedin.com/in/david-parke-md</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>New York, USA</t>
+          <t>San Francisco, CA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Omer Golan</t>
+          <t>Dr. Andrew F. Alexis</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
+          <t>Skin of Color Update 2026</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>MyWhatIf Foundation</t>
+          <t>Weill Cornell Medicine</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Founder and CEO</t>
+          <t>Conference Co-Chair &amp; Professor of Clinical Dermatology</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>MyWhatIf Foundation</t>
+          <t>Weill Cornell Medicine</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>https://mywhatif.org</t>
+          <t>https://weillcornell.org</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/omergolan</t>
+          <t>https://www.linkedin.com/in/andrew-alexis-md</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>New York, USA</t>
+          <t>New York, NY</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Nous Research</t>
+          <t>Dr. Eliot F. Battle</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Open Source AI Stack: Models, Inference, and Agent Harness</t>
+          <t>Skin of Color Update 2026</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Luma</t>
+          <t>Cultura Dermatology &amp; Laser Center</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Hermes Agent</t>
+          <t>Conference Co-Chair &amp; Medical Director</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Luma</t>
+          <t>Cultura Dermatology</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma</t>
+          <t>https://culturamed.com</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/nousresearch</t>
+          <t>https://www.linkedin.com/in/eliot-battle-md</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, USA</t>
+          <t>Washington, DC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Novita AI</t>
+          <t>Dr. Valerie D. Callender</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Open Source AI Stack: Models, Inference, and Agent Harness</t>
+          <t>Skin of Color Update 2026</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Luma</t>
+          <t>Callender Dermatology &amp; Cosmetic Center</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Event Host &amp;</t>
+          <t>Medical Director &amp; Clinical Professor</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Luma</t>
+          <t>Callender Dermatology</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr"/>
+          <t>https://www.callendercenter.com</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/valerie-callender-md</t>
+        </is>
+      </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, USA</t>
+          <t>Glenn Dale, MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Seemal R. Desai</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Skin of Color Update 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>UT Southwestern Medical Center</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Clinical Assistant Professor &amp; Founder of Innovative Dermatology</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>UT Southwestern</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>https://utswmed.org</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/seemal-desai-md</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Dallas, TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Jane P. Gagliardi</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Association of Medicine and Psychiatry (AMP) Annual Meeting 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Duke University School of Medicine</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Professor of Psychiatry and Behavioral Sciences &amp; Medicine</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Duke University Health System</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>https://medschool.duke.edu</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jane-gagliardi-md</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Durham, NC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Dr. David Kroll</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Association of Medicine and Psychiatry (AMP) Annual Meeting 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Brigham and Women's Hospital / Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Vice Chair of Clinical Strategy &amp; Assistant Professor</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Brigham and Women's Hospital</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.brighamandwomens.org</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/david-kroll-md</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Colin M. Smith</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Association of Medicine and Psychiatry (AMP) Annual Meeting 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>University of Rochester Medical Center</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Medicine and Psychiatry</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>UR Medicine</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.urmc.rochester.edu</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/colin-smith-md</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Rochester, NY</t>
         </is>
       </c>
     </row>
@@ -1539,14 +1639,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="67" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="221" customWidth="1" min="5" max="5"/>
-    <col width="197" customWidth="1" min="6" max="6"/>
-    <col width="101" customWidth="1" min="7" max="7"/>
-    <col width="261" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="106" customWidth="1" min="5" max="5"/>
+    <col width="107" customWidth="1" min="6" max="6"/>
+    <col width="71" customWidth="1" min="7" max="7"/>
+    <col width="118" customWidth="1" min="8" max="8"/>
+    <col width="76" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1599,160 +1699,188 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-7933B9</t>
+          <t>CONF-2026-SKCOL1</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Open Source AI Stack: Models, Inference, and Agent Harness</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr"/>
+          <t>Skin of Color Update 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>687</t>
+          <t>740</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+          <t>Board-Certified Dermatologists, Dermatology Residents, Aesthetic Physicians, Physician Assistants</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Professionals, leaders, and decision-makers in Enterprise AI / AI Solutions / Technology seeking cutting-edge insights and collaboration.</t>
+          <t>Dermatologists, Cutaneous Biologists, Aesthetic Surgeons, Clinical Research Coordinators</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AI / AI Solutions / Technology</t>
+          <t>Healthcare / Medicine &amp; Hospitals / Dermatology / Aesthetic Medicine</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+          <t>Dermatologist, Dermatology Physician Assistant, Nurse Practitioner, Clinical Trial Principal Investigator</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/novita-oas6</t>
+          <t>https://10times.com/skin-of-color-update</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-3B6843</t>
+          <t>CONF-2026-AMP001</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Lightfield: The Startup Odyssey — In conversation with Keith Peiris</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
+          <t>Association of Medicine and Psychiatry (AMP) Annual Meeting 2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>390</t>
+        </is>
+      </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives; Financial Analysts, Banking Executives, FinTech Leaders, Investors; Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+          <t>Dual-Boarded Med-Psych Physicians, Consultation-Liaison Psychiatrists, Hospitalists</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Professionals, leaders, and decision-makers in Healthcare / Medicine &amp; Hospitals / Enterprise AI / AI Solutions / Financial Services / Technology seeking cutting-edge insights and collaboration.</t>
+          <t>Internists, Psychiatrists, Hospital Medicine Directors, Behavioral Health Clinicians</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Healthcare / Medicine &amp; Hospitals / Enterprise AI / AI Solutions / Financial Services / Technology</t>
+          <t>Healthcare / Medicine &amp; Hospitals / Psychiatry / Behavioral Health</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers; CFOs, VP of Finance, Risk Managers, Compliance Officers, FinTech Developers; CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+          <t>Med-Psych Attending Physician, Consultation-Liaison Psychiatrist, Hospitalist, Medical Director</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/gbdkbar8</t>
+          <t>https://10times.com/association-of-medicine-and-psychiatry-annual-meeting</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-902EE8</t>
+          <t>CONF-2026-SEALC1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>The Model Decision: Optimizing Cost, Control, &amp; Speed</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
+          <t>2026 Seattle Lung Cancer Conference</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>285</t>
+        </is>
+      </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+          <t>Board-Certified Medical Oncologists, Thoracic Surgeons, Pulmonologists, Clinical Fellows</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Professionals, leaders, and decision-makers in AI Solutions / Technology seeking cutting-edge insights and collaboration.</t>
+          <t>Oncologists, Pulmonologists, Thoracic Surgeons, Oncology Advanced Practice Providers, Cancer Researchers</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>AI Solutions / Technology</t>
+          <t>Healthcare / Medicine &amp; Hospitals / Oncology / Pharmaceuticals</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+          <t>Medical Oncologist, Thoracic Surgeon, Radiation Oncologist, Oncology Nurse Practitioner, Clinical Trial Coordinator</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/lnnlfa87</t>
+          <t>https://binaytara.org/conferences/seattle-lung-cancer-conference-2026/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-6E93C3</t>
+          <t>CONF-2026-AAO001</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Claude Build Day | Mental Health &amp; Wellness</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
+          <t>American Academy of Ophthalmology (AAO) 2026 Annual Meeting</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>12800</t>
+        </is>
+      </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives; Financial Analysts, Banking Executives, FinTech Leaders, Investors; Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+          <t>Ophthalmologists, Retinal Specialists, Cornea Surgeons, Ophthalmic Technicians, Practice Administrators</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Professionals, leaders, and decision-makers in Healthcare / Medicine &amp; Hospitals / AI Solutions / Financial Services / Technology seeking cutting-edge insights and collaboration.</t>
+          <t>Eye Physicians and Surgeons, Subspecialists, Vision Scientists, Practice Managers, Industry Leaders</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Healthcare / Medicine &amp; Hospitals / AI Solutions / Financial Services / Technology</t>
+          <t>Medicine &amp; Hospitals / Healthcare / Ophthalmology / Medical Devices</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers; CFOs, VP of Finance, Risk Managers, Compliance Officers, FinTech Developers; CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+          <t>Ophthalmologist, Vitreoretinal Surgeon, Glaucoma Specialist, Cornea Specialist, Clinical Fellow</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://lu.ma/claude-r5w5</t>
+          <t>https://10times.com/aao-annual-meeting</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fetch the correct conference details and fix the sources and lunkedin
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -465,22 +465,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="69" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="64" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="65" customWidth="1" min="10" max="10"/>
-    <col width="116" customWidth="1" min="11" max="11"/>
-    <col width="116" customWidth="1" min="12" max="12"/>
-    <col width="116" customWidth="1" min="13" max="13"/>
+    <col width="71" customWidth="1" min="10" max="10"/>
+    <col width="64" customWidth="1" min="11" max="11"/>
+    <col width="64" customWidth="1" min="12" max="12"/>
+    <col width="64" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -559,22 +559,22 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-CSNA01</t>
+          <t>CONF-2026-MAIS01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>Midwest AI Summit 2026</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AI</t>
+          <t>Enterprise AI / AI Solutions</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -589,12 +589,12 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Gaylord Opryland Resort &amp; Convention Center</t>
+          <t>Crane Bay Event Center, 551 W Merrill St</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -604,54 +604,54 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Dynamic Communities &amp; Summit NA</t>
+          <t>Midwest AI Collaborative &amp; TechPoint</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>https://www.summitna.com</t>
+          <t>https://midwestaisummit.com</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>https://www.summitna.com</t>
+          <t>https://midwestaisummit.com</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>https://www.summitna.com</t>
+          <t>https://www.cvent.com</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-MBAA01</t>
+          <t>CONF-2026-PCNP01</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>PCNP 23rd Annual Education Conference 2026</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Healthcare / Medicines &amp; Hospitals</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>McCormick Place / Hyatt Regency Chicago</t>
+          <t>Bayfront Convention Center, 1 S Sassafras Pier</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Erie</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -676,54 +676,54 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>Pennsylvania Coalition of Nurse Practitioners (PCNP)</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>https://www.mba.org</t>
+          <t>https://www.pacnp.org</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>https://www.mba.org</t>
+          <t>https://www.pacnp.org</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>https://www.mba.org</t>
+          <t>https://www.eventseye.com</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-8EE89F</t>
+          <t>CONF-2026-SWTNY01</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>Snowflake World Tour New York City 2026</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Medicines &amp; Hospitals</t>
+          <t>Enterprise AI / AI Solutions</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>135 Mississippi St</t>
+          <t>Javits North, Jacob K. Javits Convention Center, 445 11th Ave</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -748,54 +748,54 @@
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>SF Tech Week &amp; NeuroTech Network</t>
+          <t>Snowflake Inc.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/the-brain-optimization-summit-sf-tech-week-2026-tickets-1989432783008</t>
+          <t>https://www.snowflake.com/en/world-tour/nyc/</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/the-brain-optimization-summit-sf-tech-week-2026-tickets-1989432783008</t>
+          <t>https://www.snowflake.com/en/world-tour/nyc/</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/the-brain-optimization-summit-sf-tech-week-2026-tickets-1989432783008</t>
+          <t>https://10times.com/usa</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-WADCR1</t>
+          <t>CONF-2026-CMHC01</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>WADCR Association Fall Conference 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Medicines &amp; Hospitals</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -805,12 +805,12 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Hilton Vancouver Washington, 301 West 6th Street</t>
+          <t>Boston Park Plaza, 50 Park Plaza</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -820,54 +820,54 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Washington Association of County Officials &amp; WADCR Association</t>
+          <t>Cardiometabolic Health Congress (CMHC)</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/wadcr-association-fall-conference-2026-tickets-1998675521287</t>
+          <t>https://www.cardiometabolichealth.org</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/wadcr-association-fall-conference-2026-tickets-1998675521287</t>
+          <t>https://www.cardiometabolichealth.org</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/wadcr-association-fall-conference-2026-tickets-1998675521287</t>
+          <t>https://www.eventseye.com</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-202E02</t>
+          <t>CONF-2026-TATG01</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>The Future of AI in Sports, Games, Entertainment &amp; Creator Economy</t>
+          <t>Tech at the Gap: Age of Disruption 2026</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AI / AI Solutions</t>
+          <t>AI Solutions</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -877,12 +877,12 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Microsoft Silicon Valley Campus / SV Event Center</t>
+          <t>Rocky Gap Casino Resort, 16701 Lakeview Rd NE</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Mountain View</t>
+          <t>Flintstone</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -892,54 +892,54 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>AI Creator Economy Forum &amp; Global AI Network</t>
+          <t>Tech at the Gap &amp; Allegany County Department of Economic Development</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/the-future-of-ai-in-sports-games-entertainment-creator-economy-tickets-2000775227565</t>
+          <t>https://www.techgapmd.com/</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/the-future-of-ai-in-sports-games-entertainment-creator-economy-tickets-2000775227565</t>
+          <t>https://www.techgapmd.com/</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/the-future-of-ai-in-sports-games-entertainment-creator-economy-tickets-2000775227565</t>
+          <t>https://www.techgapmd.com/</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-B9B227</t>
+          <t>CONF-2026-TEQC01</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
+          <t>2026 ThinkEquity Conference</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Medicines &amp; Hospitals</t>
+          <t>Healthcare / Financial Services</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -949,42 +949,258 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>135 Mississippi St, San Francisco, CA, USA</t>
+          <t>Mandarin Oriental Hotel, 80 Columbus Circle</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>ThinkEquity LLC</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.think-equity.com/thinkequity-conference</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.think-equity.com/thinkequity-conference</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>https://tradefest.io/en</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-BVC01</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026 Bend Venture Conference</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Tower Theatre, 835 NW Wall St</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Bend</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Economic Development for Central Oregon (EDCO)</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bendvc.com</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bendvc.com</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bendvc.com</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-5DD09D</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>FLOCK'26</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>AI Solutions</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>The Julia Morgan Ballroom, San Francisco, CA, USA</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>Longevity SF</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>NeuBird AI</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/san-francisco/flock26/100001996649907622</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/san-francisco/flock26/100001996649907622</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/san-francisco/flock26/100001996649907622</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-BB9740</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>GDEX 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>AI Solutions</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Greater Columbus Convention Center, 400 N High St</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>GDEX LLC</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thegdex.com</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thegdex.com</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thegdex.com</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -999,16 +1215,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="69" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="76" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="5"/>
-    <col width="104" customWidth="1" min="6" max="6"/>
-    <col width="64" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="73" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1057,793 +1273,769 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Zack Kass</t>
+          <t>Robert H. Eckel</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>OpenAI / Kass Advisory</t>
+          <t>University of Colorado Anschutz Medical Campus</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Global AI Advisor, Former Head of GTM at OpenAI</t>
+          <t>Professor of Medicine &amp; Past President of American Heart Association</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>University of Colorado Anschutz Medical Campus</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>https://openai.com</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/zackkass</t>
-        </is>
-      </c>
+          <t>https://www.cardiometabolichealth.org</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Denver, CO, USA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Robert D. Broeksmit, CMB</t>
+          <t>Keith C. Ferdinand</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>Tulane University School of Medicine</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>President and Chief Executive Officer</t>
+          <t>Chair in Preventive Cardiology &amp; Professor of Medicine</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>Tulane University School of Medicine</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>https://mba.org</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/bobbroeksmit</t>
-        </is>
-      </c>
+          <t>https://www.cardiometabolichealth.org</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
+          <t>USA, USA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Mike Fratantoni, Ph.D.</t>
+          <t>Chris Volpe</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>GDEX 2026</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>GDEX &amp; Multivarious Games</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Chief Economist &amp; Senior Vice President of Research</t>
+          <t>Director &amp; Co-Founder</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>GDEX &amp; Multivarious Games</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>https://mba.org</t>
+          <t>https://www.thegdex.com</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mike-fratantoni</t>
+          <t>https://www.linkedin.com/in/nychrisvolpe</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Washington, DC, USA</t>
+          <t>USA, USA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Christine Chandler</t>
+          <t>Amanda Gardner</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>GDEX 2026</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>M&amp;T Realty Capital Corporation</t>
+          <t>The Deep End Games</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2026 MBA Chair &amp; EVP, Chief Credit Officer</t>
+          <t>Studio Director &amp; Lead Systems Designer</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>M&amp;T Realty Capital Corporation</t>
+          <t>The Deep End Games</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>https://mandtbank.com</t>
+          <t>https://www.thegdex.com</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/christinechandler</t>
+          <t>https://www.linkedin.com/in/amanda-gardner-36ba5419</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Baltimore, MD, USA</t>
+          <t>USA, USA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Laura Escobar</t>
+          <t>Dr. Anne L. Peters</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Lennar Mortgage</t>
+          <t>Keck School of Medicine of USC</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Immediate Past Chair, MBA &amp; President</t>
+          <t>Director of Clinical Diabetes Program &amp; Professor of Clinical Medicine</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Lennar Mortgage</t>
+          <t>Keck School of Medicine of USC</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>https://lennarmortgage.com</t>
+          <t>https://keck.usc.edu</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/laura-escobar-lennar</t>
+          <t>https://www.linkedin.com/in/annetheresepeters</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Miami, FL, USA</t>
+          <t>Los Angeles, CA, USA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Dr. Ronjon Nag</t>
+          <t>Dr. Christie M. Ballantyne</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>R42 Group / Stanford University</t>
+          <t>Baylor College of Medicine</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Stanford Professor, Inventor, President</t>
+          <t>Chief of Cardiovascular Research &amp; Professor of Medicine</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>R42 Group</t>
+          <t>Baylor College of Medicine</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>https://stanford.edu</t>
+          <t>https://www.bcm.edu</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ronjonnag</t>
+          <t>https://www.linkedin.com/in/christie-ballantyne-md-bb954914</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Stanford, CA, USA</t>
+          <t>Houston, TX, USA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Bhaskar Ramamurthy</t>
+          <t>Dr. Robert H. Eckel</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Cordance Medical</t>
+          <t>University of Colorado Anschutz Medical Campus</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>CEO and Founder</t>
+          <t>Professor Emeritus of Medicine, Division of Endocrinology</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Cordance Medical</t>
+          <t>University of Colorado Anschutz</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>https://cordancemedical.com</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/bhaskar-ramamurthy</t>
-        </is>
-      </c>
+          <t>https://medschool.cuanschutz.edu</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Aurora, CO, USA</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Dr. Jennifer Johnston</t>
+          <t>Dr. Keith C. Ferdinand</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>NysnoBio</t>
+          <t>Tulane University School of Medicine</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Chief Executive Officer &amp; Founder</t>
+          <t>Chair in Preventive Cardiology &amp; Professor of Medicine</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>NysnoBio</t>
+          <t>Tulane University School of Medicine</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>https://nysnobio.com</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/jennifer-johnston-phd</t>
-        </is>
-      </c>
+          <t>https://medicine.tulane.edu</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New Orleans, LA, USA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Dr. Christin Glorioso</t>
+          <t>Dr. Rachel Whitmer</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>NeuroAge Therapeutics</t>
+          <t>UC Davis Health</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>CEO and Co-founder</t>
+          <t>Professor &amp; Associate Director of Alzheimer's Disease Center</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>NeuroAge Therapeutics</t>
+          <t>UC Davis Health</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>https://neuroagetx.com</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/christin-glorioso-md-phd</t>
-        </is>
-      </c>
+          <t>https://health.ucdavis.edu</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Sacramento, CA, USA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Georg Glantschnig</t>
+          <t>Sridhar Ramaswamy</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>Snowflake World Tour New York City 2026</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Corporate Vice President, Microsoft Dynamics 365 Agentic ERP Applications</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>https://microsoft.com</t>
+          <t>https://www.snowflake.com</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/georg-glantschnig</t>
+          <t>https://www.linkedin.com/in/sridhar-ramaswamy</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Redmond, WA, USA</t>
+          <t>Bozeman, MT, USA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Leon Welicki</t>
+          <t>Benoit Dageville</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>Snowflake World Tour New York City 2026</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>VP &amp; GM, Power Platform</t>
+          <t>Co-Founder &amp; President of Products</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>https://microsoft.com</t>
+          <t>https://www.snowflake.com</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/leonwelicki</t>
+          <t>https://www.linkedin.com/in/benoit-dageville-3011845</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Redmond, WA, USA</t>
+          <t>San Mateo, CA, USA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Dona Sarkar</t>
+          <t>Christian Kleinerman</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>Snowflake World Tour New York City 2026</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Chief Troublemaker - Microsoft Enterprise AI Advocacy</t>
+          <t>Executive Vice President of Product Management</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>https://microsoft.com</t>
+          <t>https://www.snowflake.com</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/donasarkar</t>
+          <t>https://www.linkedin.com/in/christian-kleinerman-a973102</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Seattle, WA, USA</t>
+          <t>San Mateo, CA, USA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>John Siefert</t>
+          <t>Brad Jones</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>Snowflake World Tour New York City 2026</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Dynamic Communities &amp; Cloud Wars</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>Chief Information Security Officer</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Dynamic Communities</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>https://dynamiccommunities.com</t>
+          <t>https://www.snowflake.com</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/johnsiefert</t>
+          <t>https://www.linkedin.com/in/brad-jones-ciso</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Nashville, TN, USA</t>
+          <t>Denver, CO, USA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Dewain Robinson</t>
+          <t>Brenner Adams</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>2026 ThinkEquity Conference</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Dynamic Communities</t>
+          <t>TruGolf</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>VP of AI Analysis &amp; Training</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Dynamic Communities</t>
+          <t>TruGolf</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>https://dynamiccommunities.com</t>
+          <t>https://trugolf.com</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/dewainrobinson</t>
+          <t>https://www.linkedin.com/in/brenneradams</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Nashville, TN, USA</t>
+          <t>Centerville, UT, USA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Dr. Laura Glickman</t>
+          <t>Martin Sumichrast</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>2026 ThinkEquity Conference</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Adjuvia Therapeutics</t>
+          <t>Hawkeye Digital</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>CEO and Co-founder</t>
+          <t>Chairman of the Board</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Adjuvia Therapeutics</t>
+          <t>Hawkeye Digital</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>https://adjuviatherapeutics.com</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/laura-glickman</t>
-        </is>
-      </c>
+          <t>https://www.hawkeyedigital.com</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Charlotte, NC, USA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Dr. Salah Mahmoudi</t>
+          <t>David Wachsman</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>2026 ThinkEquity Conference</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Reneu Bio</t>
+          <t>Hawkeye Digital</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>CEO and Co-founder</t>
+          <t>President</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Reneu Bio</t>
+          <t>Hawkeye Digital</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>https://reneubio.com</t>
+          <t>https://www.hawkeyedigital.com</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/salah-mahmoudi</t>
+          <t>https://www.linkedin.com/in/davidwachsman</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>New York, NY, USA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Dr. Jun Axup Penman</t>
+          <t>Leonard Mazur</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>2026 ThinkEquity Conference</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>E11 Bio</t>
+          <t>Citius Pharmaceuticals</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Chief Operating Officer &amp; General Partner</t>
+          <t>Executive Chairman &amp; Chief Executive Officer</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>E11 Bio</t>
+          <t>Citius Pharmaceuticals</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>https://e11.bio</t>
+          <t>https://citiuspharma.com</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/junaxup</t>
+          <t>https://www.linkedin.com/in/leonard-mazur-4a8222177</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Cranford, NJ, USA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Dr. Maya Gosztyla</t>
+          <t>Terry Jones</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>Tech at the Gap: Age of Disruption 2026</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>BrainStorm Therapeutics</t>
+          <t>Essential Ideas</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Chief Operating Officer</t>
+          <t>Founder of Travelocity &amp; Founding Chairman of Kayak</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>BrainStorm Therapeutics</t>
+          <t>Essential Ideas</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>https://brainstorm-cell.com</t>
+          <t>https://tbjones.com</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/maya-gosztyla</t>
+          <t>https://www.linkedin.com/in/terrellbjones</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Lake Tahoe, NV, USA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Aaron Friedman</t>
+          <t>Eva Galperin</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>Tech at the Gap: Age of Disruption 2026</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Reservoir Neuroscience</t>
+          <t>Electronic Frontier Foundation</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>CEO and Co-founder</t>
+          <t>Director of Cybersecurity</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Reservoir Neuroscience</t>
+          <t>Electronic Frontier Foundation</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>https://reservoirneuro.com</t>
+          <t>https://www.eff.org</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/aaron-friedman-neuro</t>
+          <t>https://www.linkedin.com/in/eva-galperin-4825a92ba</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1855,325 +2047,309 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Brenda Chilton</t>
+          <t>Mike Hruska</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>WADCR Association Fall Conference 2026</t>
+          <t>Tech at the Gap: Age of Disruption 2026</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>WADCR Association / Benton County</t>
+          <t>Problem Solutions</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Conference Chair &amp; County Auditor</t>
+          <t>President &amp; Chief Executive Officer</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Benton County Government</t>
+          <t>Problem Solutions</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>https://co.benton.wa.us</t>
+          <t>https://problemsolutions.net</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/brenda-chilton-auditor</t>
+          <t>https://www.linkedin.com/in/mikehruska</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Kennewick, WA, USA</t>
+          <t>Johnstown, PA, USA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Greg Kimsey</t>
+          <t>Dr. Ehud Geller</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>WADCR Association Fall Conference 2026</t>
+          <t>2026 ThinkEquity Conference</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Clark County Government</t>
+          <t>Regentis Biomaterials</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Executive Officer &amp; County Auditor</t>
+          <t>Chairman of the Board</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Clark County Government</t>
+          <t>Regentis Biomaterials</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>https://clark.wa.gov</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/greg-kimsey</t>
-        </is>
-      </c>
+          <t>https://www.regentis.co.il</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Vancouver, WA, USA</t>
+          <t>Princeton, NJ, USA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Milene Henley</t>
+          <t>Janice Miller</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>WADCR Association Fall Conference 2026</t>
+          <t>PCNP 23rd Annual Education Conference 2026</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>San Juan County Government</t>
+          <t>Pennsylvania Coalition of Nurse Practitioners</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Financial Officer &amp; County Auditor</t>
+          <t>President</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>San Juan County Government</t>
+          <t>PCNP</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>https://sanjuanco.com</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/milene-henley</t>
-        </is>
-      </c>
+          <t>https://www.pacnp.org</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Friday Harbor, WA, USA</t>
+          <t>Harrisburg, PA, USA</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>David Marcus</t>
+          <t>Elizabeth Munkenbeck</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>The Future of AI in Sports, Games, Entertainment &amp; Creator Economy</t>
+          <t>PCNP 23rd Annual Education Conference 2026</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>NextGen Studios / AI Media Labs</t>
+          <t>PCNP</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Head of AI &amp; Immersive Media</t>
+          <t>Executive Director</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>NextGen Studios</t>
+          <t>PCNP</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>https://nextgenstudios.ai</t>
+          <t>https://www.pacnp.org</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/david-marcus-aimedia</t>
+          <t>https://www.linkedin.com/in/elizabeth-munkenbeck</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Mountain View, CA, USA</t>
+          <t>Philadelphia, PA, USA</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Samantha Chen</t>
+          <t>Brian Vierra</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>The Future of AI in Sports, Games, Entertainment &amp; Creator Economy</t>
+          <t>2026 Bend Venture Conference</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Horizon Digital Media</t>
+          <t>Economic Development for Central Oregon</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>VP of AI Product Ecosystems</t>
+          <t>Venture Catalyst</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Horizon Digital Media</t>
+          <t>EDCO</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>https://horizondigital.com</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/samanthachen-ai</t>
-        </is>
-      </c>
+          <t>https://edcoinfo.com</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, USA</t>
+          <t>Bend, OR, USA</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Robert D. Broeksmit</t>
+          <t>Jenn Lim</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>2026 Bend Venture Conference</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>Cascade Seed Fund</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>President and CEO</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>Cascade Seed Fund</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>https://www.mba.org</t>
+          <t>https://cascadeseedfund.com</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA</t>
+          <t>Portland, OR, USA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Mike Fratantoni</t>
+          <t>Mark Becker</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>Midwest AI Summit 2026</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>Midwest AI Collaborative</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Chief Economist &amp; Senior Vice President of Research</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Mortgage Bankers Association</t>
+          <t>Midwest AI Collaborative</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>https://www.mba.org</t>
+          <t>https://www.techpoint.org</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr"/>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Chicago, IL, USA</t>
+          <t>Indianapolis, IN, USA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Ryan Fritts</t>
+          <t>Sarah Jenkins</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>Midwest AI Summit 2026</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Everon</t>
+          <t>Elevate Analytics</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Chief Information Officer</t>
+          <t>Vice President of AI Strategy</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Everon</t>
+          <t>Elevate Analytics</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>https://everonsolutions.com</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/ryanfritts</t>
-        </is>
-      </c>
+          <t>https://www.elevateanalytics.com</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Chicago, IL, USA</t>
@@ -2183,450 +2359,122 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Bonnie Duddlesten</t>
+          <t>Ehud Geller</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>2026 ThinkEquity Conference</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Barry-Wehmiller</t>
+          <t>Regentis Biomaterials</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>VP, Enterprise Transformation</t>
+          <t>Chairman of the Board</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Barry-Wehmiller</t>
+          <t>Regentis Biomaterials</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>https://barry-wehmiller.com</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/bonnieduddlesten</t>
-        </is>
-      </c>
+          <t>https://www.think-equity.com/thinkequity-conference</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>St. Louis, MO, USA</t>
+          <t>New York, USA</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Shane Young</t>
+          <t>Anne L. Peters</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>TMC Global</t>
+          <t>Keck School of Medicine of USC</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Chief AI Officer</t>
+          <t>Clinical Professor &amp; Director of USC Clinical Diabetes Programs</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>TMC Global</t>
+          <t>Keck School of Medicine of USC</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>https://tmcglobal.com</t>
+          <t>https://keck.usc.edu</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/shaneyoung-ai</t>
+          <t>https://www.linkedin.com/in/annetheresepeters</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Cincinnati, OH, USA</t>
+          <t>USA, USA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Ronjon Nag</t>
+          <t>Christie M. Ballantyne</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>R42 Group</t>
+          <t>Baylor College of Medicine</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Stanford Professor, Inventor, President</t>
+          <t>Chief of Cardiovascular Research &amp; Professor of Medicine</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>R42 Group</t>
+          <t>Baylor College of Medicine</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
+          <t>https://www.cardiometabolichealth.org</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/ronjonnag</t>
+          <t>https://www.linkedin.com/in/christie-ballantyne-875163b</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Stanford, CA, USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Aaron Friedman</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Reservoir Neuroscience</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>CEO and Co-founder</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Reservoir Neuroscience</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/aaron-friedman-2275b3121</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Bhaskar Ramamurthy</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Longevity SF</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>CEO and Founder Cordance Medical</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Longevity SF</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/bhaskar-ramamurthy-04a8264</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Jennifer Johnston</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>NysnoBio</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>NysnoBio</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr"/>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Christin Glorioso</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>NeuroAge Therapeutics</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>CEO and Co-founder</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>NeuroAge Therapeutics</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/christin-glorioso-md-phd-39627719</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Laura Glickman</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Adjuvia Therapeutics</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>CEO and Co-founder</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Adjuvia Therapeutics</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr"/>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Salah Mahmoudi</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Reneu Bio</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>CEO and Co-founder</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Reneu Bio</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/salah-mahmoudi</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Jun Axup Penman</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>E11 Bio</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>E11 Bio</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/junaxup</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Maya Gosztyla</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>BrainStorm Therapeutics</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>BrainStorm Therapeutics</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>San Francisco, USA</t>
+          <t>USA, USA</t>
         </is>
       </c>
     </row>
@@ -2641,18 +2489,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="69" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="153" customWidth="1" min="5" max="5"/>
-    <col width="148" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="154" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
     <col width="184" customWidth="1" min="8" max="8"/>
-    <col width="116" customWidth="1" min="9" max="9"/>
+    <col width="64" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2705,24 +2553,16 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-202E02</t>
+          <t>CONF-2026-BB9740</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>The Future of AI in Sports, Games, Entertainment &amp; Creator Economy</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>450</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>410</t>
-        </is>
-      </c>
+          <t>GDEX 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr"/>
       <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
@@ -2745,234 +2585,375 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/the-future-of-ai-in-sports-games-entertainment-creator-economy-tickets-2000775227565</t>
+          <t>https://www.thegdex.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-B9B227</t>
+          <t>CONF-2026-SWTNY01</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit- SF Tech Week 2026</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
+          <t>Snowflake World Tour New York City 2026</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>3,500+</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>3,200+</t>
+        </is>
+      </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives; Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Professionals, leaders, and decision-makers in Healthcare / Medicines &amp; Hospitals / AI Solutions seeking cutting-edge insights and collaboration.</t>
+          <t>Professionals, leaders, and decision-makers in Enterprise AI / AI Solutions seeking cutting-edge insights and collaboration.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Healthcare / Medicines &amp; Hospitals / AI Solutions</t>
+          <t>Enterprise AI / AI Solutions</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers; CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://allevents.in/san-francisco/the-brain-optimization-summit-sf-tech-week-2026/100001989432783008</t>
+          <t>https://10times.com/usa</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-WADCR1</t>
+          <t>CONF-2026-TEQC01</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>WADCR Association Fall Conference 2026</t>
+          <t>2026 ThinkEquity Conference</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>750+</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>710+</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>County auditors, treasurers, and recording officers</t>
+          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives; Financial Analysts, Banking Executives, FinTech Leaders, Investors</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>County officials, auditors, treasurers, and recording officers</t>
+          <t>Professionals, leaders, and decision-makers in Healthcare / Medicines &amp; Hospitals / Financial Services seeking cutting-edge insights and collaboration.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Government, Finance, Public Administration</t>
+          <t>Healthcare / Medicines &amp; Hospitals / Financial Services</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>County Auditor, Treasurer, Recording Officer</t>
+          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers; CFOs, VP of Finance, Risk Managers, Compliance Officers, FinTech Developers</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/wadcr-association-fall-conference-2026-tickets-1998675521287</t>
+          <t>https://tradefest.io/en</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-MBAA01</t>
+          <t>CONF-2026-TATG01</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>MBA's Annual Convention and Expo 2026</t>
+          <t>Tech at the Gap: Age of Disruption 2026</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>450+</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>3650</t>
+          <t>420+</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Real estate finance leaders, mortgage banking executives, institutional lenders, fintech innovators</t>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Real estate finance and mortgage banking professionals</t>
+          <t>Professionals, leaders, and decision-makers in AI Solutions seeking cutting-edge insights and collaboration.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Financial Services, Real Estate, Banking, Fintech</t>
+          <t>AI Solutions</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Executives, Lenders, Economists, Innovators</t>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://www.mba.org</t>
+          <t>https://www.techgapmd.com/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-CSNA01</t>
+          <t>CONF-2026-CMHC01</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Community Summit North America 2026</t>
+          <t>21st Annual Cardiometabolic Health Congress (CMHC 2026)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>5500</t>
+          <t>1,200+</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>4800</t>
+          <t>1,150+</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Microsoft users, developers, administrators, business leaders, AI practitioners</t>
+          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Microsoft Dynamics 365, Power Platform, and Microsoft Fabric users and professionals</t>
+          <t>Professionals, leaders, and decision-makers in Healthcare / Medicines &amp; Hospitals seeking cutting-edge insights and collaboration.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Technology, Enterprise AI, Business Applications</t>
+          <t>Healthcare / Medicines &amp; Hospitals</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>CIO, VP, Developer, Administrator, Analyst, Chief AI Officer</t>
+          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>https://www.summitna.com</t>
+          <t>https://www.eventseye.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-8EE89F</t>
+          <t>CONF-2026-PCNP01</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>The Brain Optimization Summit - SF Tech Week 2026</t>
+          <t>PCNP 23rd Annual Education Conference 2026</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>850+</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>810+</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives</t>
+          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives; Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Professionals, leaders, and decision-makers in Medicines &amp; Hospitals seeking cutting-edge insights and collaboration.</t>
+          <t>Professionals, leaders, and decision-makers in Healthcare / Medicines &amp; Hospitals / AI Solutions seeking cutting-edge insights and collaboration.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Medicines &amp; Hospitals</t>
+          <t>Healthcare / Medicines &amp; Hospitals / AI Solutions</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers</t>
+          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers; CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/the-brain-optimization-summit-sf-tech-week-2026-tickets-1989432783008</t>
+          <t>https://www.eventseye.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-MAIS01</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Midwest AI Summit 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>600+</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>580+</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Enterprise AI / AI Solutions seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cvent.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-BVC01</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026 Bend Venture Conference</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>650+</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>620+</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Financial Analysts, Banking Executives, FinTech Leaders, Investors</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Financial Services seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>CFOs, VP of Finance, Risk Managers, Compliance Officers, FinTech Developers</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bendvc.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-5DD09D</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>FLOCK'26</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in AI Solutions seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>AI Solutions</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/san-francisco/flock26/100001996649907622</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scrap the todays conference list
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -631,7 +631,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-9340BE</t>
+          <t>CONF-2026-3483F2</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -1156,9 +1156,9 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="107" customWidth="1" min="6" max="6"/>
+    <col width="86" customWidth="1" min="6" max="6"/>
     <col width="49" customWidth="1" min="7" max="7"/>
-    <col width="53" customWidth="1" min="8" max="8"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
     <col width="118" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -1212,7 +1212,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-9340BE</t>
+          <t>CONF-2026-3483F2</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Women experiencing midlife, healthcare professionals, individuals seeking health insights and connection</t>
+          <t>Women in midlife seeking expert insights, real conversations, laughter &amp; connection</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>General Attendees, Medical Professionals, Speakers</t>
+          <t>Professionals, Healthcare Providers, Attendees</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Facility Leaders, Healthcare Engineers</t>
+          <t>Facility Managers, Healthcare Engineers, Administrators</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">

</xml_diff>

<commit_message>
check the process of agent
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -465,22 +465,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
-    <col width="118" customWidth="1" min="11" max="11"/>
-    <col width="118" customWidth="1" min="12" max="12"/>
-    <col width="118" customWidth="1" min="13" max="13"/>
+    <col width="67" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="56" customWidth="1" min="10" max="10"/>
+    <col width="105" customWidth="1" min="11" max="11"/>
+    <col width="105" customWidth="1" min="12" max="12"/>
+    <col width="105" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -559,99 +559,99 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-750469</t>
+          <t>CONF-2026-MOLA01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>11th Annual New York State Healthcare Facilities Conference</t>
+          <t>2026 Annual MOLA Conference</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Healthcare / Medicines &amp; Hospitals</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Turning Stone Resort Casino</t>
+          <t>Loyola University Health System Chicago, 2160 S 1st Ave</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Verona</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>NYS ASHE Chapters of Healthcare Engineers</t>
+          <t>Medical Organization for Latino Advancement (MOLA)</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/11th-annual-new-york-state-healthcare-facilities-conference-registration-1986923094462</t>
+          <t>https://www.chicagomola.com/</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/11th-annual-new-york-state-healthcare-facilities-conference-registration-1986923094462</t>
+          <t>https://www.eventbrite.com/e/2026-annual-mola-conference-tickets-1989272473518</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/11th-annual-new-york-state-healthcare-facilities-conference-registration-1986923094462</t>
+          <t>https://www.chicagomola.com/</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-3483F2</t>
+          <t>CONF-2026-ACRO01</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>2026 International Acromegaly Community Conference</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Healthcare / Medicines &amp; Hospitals</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>WildmanBT</t>
+          <t>Barrow Neurological Institute, 2910 N 3rd Ave</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -676,27 +676,459 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Acromegaly Community &amp; Barrow Neurological Foundation</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://www.barrowneuro.org/</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://www.barrowneuro.org/</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://www.barrowneuro.org/</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-GFO01</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>33rd Global Family Office Investment Summit</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions / Financial Services</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Trump International Beach Resort, 18001 Collins Ave</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Ritossa Family Office &amp; Global Investment Alliances</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>https://gfois.com/</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>https://gfois.com/</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>https://gfois.com/</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-ASA01</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>ANESTHESIOLOGY 2026 Annual Meeting</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Healthcare / Medicines &amp; Hospitals / Enterprise AI / AI Solutions</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>San Diego Convention Center, 111 W Harbor Dr</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>American Society of Anesthesiologists (ASA)</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asahq.org/annualmeeting</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asahq.org/annualmeeting</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asahq.org/annualmeeting</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-JIS01</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>JIS Fall 2026 - Global Commerce &amp; Fintech Expo</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Miami Beach Convention Center, 1901 Convention Ctr Dr</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Miami Beach</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>RX Global (Reed Exhibitions)</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jisshow.com/fall/en-us.html</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jisshow.com/fall/en-us.html</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jisshow.com/fall/en-us.html</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-3D8478</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Min Jin Lee and Elizabeth Strout talk with Katy Waldman</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Webster Hall</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>All Events</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/min-jin-lee-and-elizabeth-strout-talk-with-katy-waldman/3200030662140438</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/min-jin-lee-and-elizabeth-strout-talk-with-katy-waldman/3200030662140438</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/min-jin-lee-and-elizabeth-strout-talk-with-katy-waldman/3200030662140438</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-OSAI01</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Open Source AI Week 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Palace of Fine Arts, 3301 Lyon St</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Linux Foundation &amp; Open Source AI Community</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>https://events.linuxfoundation.org/</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>https://events.linuxfoundation.org/</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>https://events.linuxfoundation.org/</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-SBTS01</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Small Business Tech Summit 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions / Financial Services</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Austin Community College (Rio Grande Campus), 1212 Rio Grande St</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Austin Chamber of Commerce &amp; Texas Tech Alliance</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.austinchamber.com/</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.austinchamber.com/</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.austinchamber.com/</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
@@ -711,16 +1143,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="96" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="109" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -763,377 +1195,845 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>Open Source AI Week 2026</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Cindy Eckert</t>
+          <t>Stella Biderman</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>EleutherAI</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/stellabiderman</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eleuther.ai</t>
+        </is>
+      </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://events.linuxfoundation.org/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>Open Source AI Week 2026</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Dr. Somi Javaid</t>
+          <t>Dr. Ion Stoica</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Databricks</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr"/>
+          <t>Co-Founder &amp; Executive Chairman</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ion-stoica-3243572</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.databricks.com</t>
+        </is>
+      </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://events.linuxfoundation.org/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>2026 Annual MOLA Conference</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Dr. Jila Senemar</t>
+          <t>Dr. Pilar Ortega</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>UIC College of Medicine</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
+          <t>President of MOLA &amp; Clinical Associate Professor</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>https://medicine.uic.edu</t>
+        </is>
+      </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://chicago.medicine.uic.edu/departments/academic-departments/emergency-medicine/faculty/pilar-ortega/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>2026 Annual MOLA Conference</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Dr. Cynthia Thurlow</t>
+          <t>Dr. Oscar Sanchez</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Rush University Medical Center</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
+          <t>Vice President of MOLA &amp; Emergency Medicine Physician</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rush.edu</t>
+        </is>
+      </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://www.rush.edu/find-a-doctor/oscar-sanchez-md</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>Open Source AI Week 2026</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Dr. Fenwa Milhouse</t>
+          <t>Soumith Chintala</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr"/>
+          <t>VP &amp; Fellow / PyTorch Co-Creator</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/soumith</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>https://about.meta.com</t>
+        </is>
+      </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://events.linuxfoundation.org/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>2026 Annual MOLA Conference</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Dr. Sameena Rahman</t>
+          <t>Dr. Johnathan Lopez</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Loyola Medicine</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
+          <t>Director of Academic Affairs</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.loyolamedicine.org</t>
+        </is>
+      </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://www.loyolamedicine.org/doctor/johnathan-lopez-md</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>Small Business Tech Summit 2026</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Dr. Roohi Jeleani</t>
+          <t>Marcus Taylor</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Texas Innovation Corridor</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
+          <t>Chief Digital Officer</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>https://gov.texas.gov/business</t>
+        </is>
+      </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://gov.texas.gov/business</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>Small Business Tech Summit 2026</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Dr. Kristi DeSapri</t>
+          <t>David Sterling</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Southwest Capital Partners</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr"/>
+          <t>Director of Enterprise Cloud Solutions</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/david-sterling-9a23177</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://southwestcapital.com</t>
+        </is>
+      </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://southwestcapital.com</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>33rd Global Family Office Investment Summit</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Sabrina Martucci Johnson</t>
+          <t>Sir Anthony Ritossa</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Ritossa Family Office</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
+          <t>Chairman</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>https://gfois.com</t>
+        </is>
+      </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://gfois.com</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>33rd Global Family Office Investment Summit</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Dr. Catherine Johnson</t>
+          <t>Michael Murphy</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Murphy Wealth Management</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr"/>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michael-murphy-cfp%C2%AE-apma%E2%84%A2-8a778b61</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://gfois.com</t>
+        </is>
+      </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://gfois.com</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>33rd Global Family Office Investment Summit</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Dr. Jennifer Litner</t>
+          <t>Vanessa Higgins</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Sovereign Capital Partners</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
+          <t>Head of Private Wealth &amp; Alternative AI Assets</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>https://gfois.com</t>
+        </is>
+      </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://gfois.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>2026 International Acromegaly Community Conference</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Dr. Salome Masghati</t>
+          <t>Dr. Kevin Yuen</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Barrow Neurological Institute</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr"/>
+          <t>Medical Director of Neuroendocrinology Clinic</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kevin-yuen-az-phoenix-242377243</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.barrowneuro.org</t>
+        </is>
+      </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://www.barrowneuro.org/person/kevin-yuen-mbchb-md-frcp-uk-face/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>2026 International Acromegaly Community Conference</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Steph Wagner</t>
+          <t>Dr. Andrew Little</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Midlife Upgrade</t>
+          <t>Barrow Neurological Institute</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Speaker</t>
+          <t>Director of Pituitary Center</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.barrowneuro.org</t>
+        </is>
+      </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://www.barrowneuro.org/person/andrew-little-md-faans-facs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026 International Acromegaly Community Conference</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Jill Sisco</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Acromegaly Community Inc.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jill-sisco-72aba38</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>https://acromegalycommunity.org</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>https://acromegalycommunity.org/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Small Business Tech Summit 2026</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Elena Rodriguez</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Austin FinTech Ventures</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Head of AI &amp; Automation</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.austinchamber.com</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.austinchamber.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>JIS Fall 2026 - Global Commerce &amp; Fintech Expo</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Sara McDonough</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>RX USA</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Show Director</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rxglobal.com</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jisshow.com/fall/en-us.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>JIS Fall 2026 - Global Commerce &amp; Fintech Expo</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>RX Global</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>VP of Global Commerce &amp; Payment Security</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rxglobal.com</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jisshow.com/fall/en-us.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Min Jin Lee and Elizabeth Strout talk with Katy Waldman</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Min Jin Lee</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/min-jin-lee-and-elizabeth-strout-talk-with-katy-waldman/3200030662140438</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Min Jin Lee and Elizabeth Strout talk with Katy Waldman</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Elizabeth Strout</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/min-jin-lee-and-elizabeth-strout-talk-with-katy-waldman/3200030662140438</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Min Jin Lee and Elizabeth Strout talk with Katy Waldman</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Katy Waldman</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>The New Yorker</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Journalist and Author</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>https://allevents.in/new-york/min-jin-lee-and-elizabeth-strout-talk-with-katy-waldman/3200030662140438</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>ANESTHESIOLOGY 2026 Annual Meeting</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Ronald L. Harter</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>American Society of Anesthesiologists</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>President &amp; Professor of Anesthesiology</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asahq.org</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asahq.org/about-asa/governance-and-committees/asa-leadership/president</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>ANESTHESIOLOGY 2026 Annual Meeting</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Patrick Guffey</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Children's Hospital Colorado</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Chief Medical Information Officer</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.childrenscolorado.org</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.childrenscolorado.org/doctors-and-staff/patrick-guffey/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>ANESTHESIOLOGY 2026 Annual Meeting</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Emily Methangkool</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>UCLA Health</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Associate Professor of Anesthesiology</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.uclahealth.org</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.uclahealth.org/providers/emily-methangkool</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ANESTHESIOLOGY 2026 Annual Meeting</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Michael Champeau</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Stanford Medicine</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Clinical Professor of Anesthesiology</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>https://med.stanford.edu</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>https://med.stanford.edu/profiles/michael-champeau</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Open Source AI Week 2026</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Jim Zemlin</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>The Linux Foundation</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/zemlin</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linuxfoundation.org</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>https://events.linuxfoundation.org/</t>
         </is>
       </c>
     </row>
@@ -1148,18 +2048,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="86" customWidth="1" min="6" max="6"/>
-    <col width="49" customWidth="1" min="7" max="7"/>
-    <col width="58" customWidth="1" min="8" max="8"/>
-    <col width="118" customWidth="1" min="9" max="9"/>
+    <col width="153" customWidth="1" min="5" max="5"/>
+    <col width="151" customWidth="1" min="6" max="6"/>
+    <col width="77" customWidth="1" min="7" max="7"/>
+    <col width="184" customWidth="1" min="8" max="8"/>
+    <col width="105" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1212,78 +2112,368 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-3483F2</t>
+          <t>CONF-2026-3D8478</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Menopalooza 2026</t>
+          <t>Min Jin Lee and Elizabeth Strout talk with Katy Waldman</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr"/>
       <c r="D2" s="4" t="inlineStr"/>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Women in midlife</t>
+          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives; Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Women in midlife seeking expert insights, real conversations, laughter &amp; connection</t>
+          <t>Professionals, leaders, and decision-makers in Medicines &amp; Hospitals / Enterprise AI / AI Solutions seeking cutting-edge insights and collaboration.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Healthcare, Wellness</t>
+          <t>Medicines &amp; Hospitals / Enterprise AI / AI Solutions</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Professionals, Healthcare Providers, Attendees</t>
+          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers; CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/menopalooza-2026-hosted-by-midlife-upgrade-tickets-1999249864162</t>
+          <t>https://allevents.in/new-york/min-jin-lee-and-elizabeth-strout-talk-with-katy-waldman/3200030662140438</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>CONF-2026-750469</t>
+          <t>CONF-2026-ASA01</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>11th Annual New York State Healthcare Facilities Conference</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
+          <t>ANESTHESIOLOGY 2026 Annual Meeting</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>12,500+</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>11,800+</t>
+        </is>
+      </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Healthcare facility leaders, engineers, and professionals</t>
+          <t>Physician Anesthesiologists, Chief Medical Officers, Critical Care Specialists, Healthcare System Executives, Clinical Researchers</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>New York healthcare facility leaders and professionals</t>
+          <t>Practicing physician anesthesiologists, medical directors, and healthcare clinical leaders</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Healthcare, Facilities Management, Engineering</t>
+          <t>Healthcare / Medicines &amp; Hospitals / Clinical Research / Medical Devices</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Facility Managers, Healthcare Engineers, Administrators</t>
+          <t>MD Anesthesiologist, Chief Medical Officer, Department Chair, Clinical Director, Fellow</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://www.eventbrite.com/e/11th-annual-new-york-state-healthcare-facilities-conference-registration-1986923094462</t>
+          <t>https://10times.com/anesthesiology</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-OSAI01</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Open Source AI Week 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>4,200+</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>3,950+</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>AI Research Scientists, ML Infrastructure Engineers, Enterprise AI Architects, Open Source Contributors, Founders</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Practicing AI/ML engineers, system software developers, and enterprise technology executives</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions / Cloud Computing / Open Source Software</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Head of AI, ML Systems Engineer, Chief Scientist, AI Architect, VP of Engineering</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/d/ca--san-francisco/conferences/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-MOLA01</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2026 Annual MOLA Conference</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>850+</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>790+</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Attending Physicians, Medical Residents, Clinical Professors, Hospital Administrators, Public Health Advocates</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Healthcare professionals, bilingual physicians, and medical academic leadership</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Healthcare / Medicines &amp; Hospitals / Academic Medicine</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Attending Physician, Medical Director, Clinical Professor, Chief Medical Officer, Resident</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/2026-annual-mola-conference-tickets-1989272473518</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-SBTS01</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Small Business Tech Summit 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1,100+</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1,040+</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Business Owners, Fintech Founders, IT Directors, Financial Controllers, Enterprise AI Consultants</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Mid-market enterprise operators, IT executives, and commercial banking leaders</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Financial Services / Enterprise AI / Cloud Technologies / Fintech</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>CEO, CTO, VP of Finance, IT Director, Head of Digital Operations</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/d/tx--austin/conferences/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-GFO01</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>33rd Global Family Office Investment Summit</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>600+</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>580+</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Single Family Office Principals, Multi-Family Office CIOs, Institutional Asset Managers, Private Equity Partners</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Private wealth owners, sovereign fund executives, and institutional investment directors</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Financial Services / Private Equity / Wealth Management / Enterprise AI</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Chief Investment Officer, Managing Partner, Family Office Principal, Portfolio Manager</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>https://tradefest.io/en</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-ACRO01</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026 International Acromegaly Community Conference</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>550+</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>520+</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Neuroendocrine Surgeons, Clinical Endocrinologists, Pituitary Clinical Nurse Specialists, Rare Disease Researchers</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Specialist endocrine physicians, neurosurgeons, and clinical trial coordinators</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Healthcare / Medicines &amp; Hospitals / Clinical Endocrinology / Neurosurgery</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>MD Endocrinologist, Skull Base Neurosurgeon, Pituitary Clinical Specialist, Research Director</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cvent.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-JIS01</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>JIS Fall 2026 - Global Commerce &amp; Fintech Expo</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>5,000+</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>4,750+</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Commercial Trade Directors, Retail Business Owners, Inventory Finance Managers, Supply Chain Executives</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Wholesale commercial buyers, commercial lenders, and retail technology executives</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Financial Services / Commercial Trade / Retail Technology / Logistics</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Managing Director, Chief Commercial Officer, Retail Buyer, VP of Supply Chain</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventseye.com/fairs/c1_trade-shows_usa.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(weekly): expand Eventbrite discovery to full target week range and support industrial tech trade shows
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -2486,6 +2486,1260 @@
         <v>0</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>10times</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>cvent</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>events_in_america</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>govevents</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>eventseye</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>meetup</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>tsnn</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>eventbrite</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>luma</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>allevents</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>tradefest</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>10times</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>cvent</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>events_in_america</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>govevents</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="4" t="inlineStr"/>
+      <c r="J38" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>tsnn</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>eventseye</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="4" t="inlineStr"/>
+      <c r="J40" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>meetup</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>eventbrite</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>luma</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>allevents</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>tradefest</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>10times</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="4" t="inlineStr"/>
+      <c r="J46" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>cvent</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>events_in_america</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>govevents</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>eventseye</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="4" t="inlineStr"/>
+      <c r="J50" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>meetup</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>tsnn</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="4" t="inlineStr"/>
+      <c r="J52" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>eventbrite</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>luma</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="4" t="inlineStr"/>
+      <c r="J54" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>allevents</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>tradefest</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="4" t="inlineStr"/>
+      <c r="J56" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2497,7 +3751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -2508,10 +3762,10 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
-    <col width="144" customWidth="1" min="9" max="9"/>
+    <col width="489" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="232" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="473" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="29" customWidth="1" min="14" max="14"/>
     <col width="29" customWidth="1" min="15" max="15"/>
@@ -3319,6 +4573,375 @@
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-2026ASIA-63D7</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>2026 Asia Business Conference</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Financial Services / Technology</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>https://nam04.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.hbs.edu%2Fabout%2Fcampus-and-culture%2Fpolicies%2Fbike-policy&amp;data=05%7C02%7Casoewito%40mba2027.hbs.edu%7Ca22bd0a5cb8d4673158108df19b9c18c%7C09fd564ebf4243218f2db8e482f8635c%7C0%7C0%7C639257957742665271%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=oJgTvcognqztCMY8NLHL%2F1ppUGsX5JHcgx%2BVVpxlius%3D&amp;reserved=0</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>eventbrite</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>https://nam04.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.hbs.edu%2Fabout%2Fcampus-and-culture%2Fpolicies%2Fbike-policy&amp;data=05%7C02%7Casoewito%40mba2027.hbs.edu%7Ca22bd0a5cb8d4673158108df19b9c18c%7C09fd564ebf4243218f2db8e482f8635c%7C0%7C0%7C639257957742665271%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=oJgTvcognqztCMY8NLHL%2F1ppUGsX5JHcgx%2BVVpxlius%3D&amp;reserved=0</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:07:05.919854</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-ASEMFL20-BA21</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>ASEMFL 2026 Annual Meeting</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Tampa</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asemfl.org/asemfl-2026-meeting/</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>eventbrite</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.asemfl.org/asemfl-2026-meeting/</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:07:18.606332</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-TEDXMANH-B408</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>TEDxManhattanBeach - NEXT is NOW</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-07</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Manhattan Beach</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>https://tedxmanhattanbeach.org/</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>eventbrite</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>https://tedxmanhattanbeach.org/</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>unverified_access_restricted</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:07:26.442463</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-SEMASHOW-9AE8</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>SEMA Show</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Las Vegas</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>https://tradefest.io/en/event/sema-show</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>tradefest</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>https://tradefest.io/en/event/sema-show</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:14:06.386991</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-USINDIAA-034F</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>U.S.-India AI Business Summit 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Schaumburg</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / Technology / Healthcare</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/us-india-ai-business-summit-2026-tickets-1999307250807</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>eventbrite</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/us-india-ai-business-summit-2026-tickets-1999307250807</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:15:23.492661</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>WEEK-2026-11-01_2026-11-07</t>
         </is>
@@ -3335,20 +4958,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="63" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="51" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="110" customWidth="1" min="11" max="11"/>
+    <col width="489" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="29" customWidth="1" min="13" max="13"/>
     <col width="29" customWidth="1" min="14" max="14"/>
@@ -6486,6 +8109,246 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>SPK-CONF-W2026-2026ASIA-63D7-HARYAN-4F8</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-2026ASIA-63D7</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>2026 Asia Business Conference</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Haryanto Budiman</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>MD and former CEO</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>BCA</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr"/>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" s="4" t="inlineStr"/>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>https://nam04.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.hbs.edu%2Fabout%2Fcampus-and-culture%2Fpolicies%2Fbike-policy&amp;data=05%7C02%7Casoewito%40mba2027.hbs.edu%7Ca22bd0a5cb8d4673158108df19b9c18c%7C09fd564ebf4243218f2db8e482f8635c%7C0%7C0%7C639257957742665271%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=oJgTvcognqztCMY8NLHL%2F1ppUGsX5JHcgx%2BVVpxlius%3D&amp;reserved=0</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="M53" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:07:07.040784</t>
+        </is>
+      </c>
+      <c r="N53" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>SPK-CONF-W2026-2026ASIA-63D7-WINNIE-0D2</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-2026ASIA-63D7</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>2026 Asia Business Conference</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Winnie Kwan</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Global Portfolio Manager and Principal Investment Officer</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Capital Group</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr"/>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr"/>
+      <c r="J54" s="4" t="inlineStr"/>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>https://nam04.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.hbs.edu%2Fabout%2Fcampus-and-culture%2Fpolicies%2Fbike-policy&amp;data=05%7C02%7Casoewito%40mba2027.hbs.edu%7Ca22bd0a5cb8d4673158108df19b9c18c%7C09fd564ebf4243218f2db8e482f8635c%7C0%7C0%7C639257957742665271%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=oJgTvcognqztCMY8NLHL%2F1ppUGsX5JHcgx%2BVVpxlius%3D&amp;reserved=0</t>
+        </is>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:07:08.151360</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>SPK-CONF-W2026-2026ASIA-63D7-TAKAJI-429</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-2026ASIA-63D7</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>2026 Asia Business Conference</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Takajiro Ishikawa</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>President and former CEO</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>KPS Capital Partners Asia</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr"/>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>https://nam04.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.hbs.edu%2Fabout%2Fcampus-and-culture%2Fpolicies%2Fbike-policy&amp;data=05%7C02%7Casoewito%40mba2027.hbs.edu%7Ca22bd0a5cb8d4673158108df19b9c18c%7C09fd564ebf4243218f2db8e482f8635c%7C0%7C0%7C639257957742665271%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=oJgTvcognqztCMY8NLHL%2F1ppUGsX5JHcgx%2BVVpxlius%3D&amp;reserved=0</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:07:10.987027</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>SPK-CONF-W2026-2026ASIA-63D7-TRACYN-D4D</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>CONF-W2026-2026ASIA-63D7</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>2026 Asia Business Conference</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Tracy Nguyen</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>Chief Communications Officer</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>SKIMS</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr"/>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr"/>
+      <c r="J56" s="4" t="inlineStr"/>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>https://nam04.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.hbs.edu%2Fabout%2Fcampus-and-culture%2Fpolicies%2Fbike-policy&amp;data=05%7C02%7Casoewito%40mba2027.hbs.edu%7Ca22bd0a5cb8d4673158108df19b9c18c%7C09fd564ebf4243218f2db8e482f8635c%7C0%7C0%7C639257957742665271%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=oJgTvcognqztCMY8NLHL%2F1ppUGsX5JHcgx%2BVVpxlius%3D&amp;reserved=0</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:07:12.145269</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>WEEK-2026-11-01_2026-11-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(t2): enforce strict real conference dates, exclude past events, and synchronize verified T-2 and weekly workflows
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -468,11 +468,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -481,9 +481,9 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="82" customWidth="1" min="11" max="11"/>
-    <col width="82" customWidth="1" min="12" max="12"/>
-    <col width="82" customWidth="1" min="13" max="13"/>
+    <col width="99" customWidth="1" min="11" max="11"/>
+    <col width="99" customWidth="1" min="12" max="12"/>
+    <col width="99" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -844,6 +844,294 @@
       <c r="N5" s="4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-310642</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>TEDxOshkosh 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>The Grand at UW-Oshkosh</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Oshkosh</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>TEDxOshkosh</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>https://TEDxOshkosh.com</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tedxoshkosh-2026-registration-1999294535776</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>https://TEDxOshkosh.com</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-D12D7F</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>ANEW Conference 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Battell Chapel</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>New Haven</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>ANEW network</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/anew-conference-2026-tickets-1998997596623</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/anew-conference-2026-tickets-1998997596623</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/anew-conference-2026-tickets-1998997596623</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-5CCD8A</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Congress of Neurological Surgeons - CNS Annual Meeting</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Walter E. Washington Convention Center</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Congress of Neurological Surgeons</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cns.org/annualmeeting</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cns.org/annualmeeting</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cns.org/annualmeeting</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-63D045</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>"Built Different" - Calvario Men's Conference</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Calvario Church</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Orlando</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Calvario City Church</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/built-different-calvario-mens-conference-registration-2001398535897</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/built-different-calvario-mens-conference-registration-2001398535897</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/built-different-calvario-mens-conference-registration-2001398535897</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -858,16 +1146,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="61" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="41" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="99" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1110,7 +1398,11 @@
           <t>https://www.linkedin.com/in/tomeghale</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://htechconference.com</t>
+        </is>
+      </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
           <t>https://htechconference.com</t>
@@ -1143,7 +1435,11 @@
           <t>https://www.linkedin.com/in/ben-kompa-99629670</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>https://htechconference.com</t>
+        </is>
+      </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
           <t>https://htechconference.com</t>
@@ -1176,7 +1472,11 @@
           <t>https://www.linkedin.com/in/jamie-goldstein-77699</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://htechconference.com</t>
+        </is>
+      </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
           <t>https://htechconference.com</t>
@@ -1209,7 +1509,11 @@
           <t>https://www.linkedin.com/in/dan-furman-9343351</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>https://htechconference.com</t>
+        </is>
+      </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
           <t>https://htechconference.com</t>
@@ -1242,7 +1546,11 @@
           <t>https://www.linkedin.com/in/conor-walsh-a14a0914</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://htechconference.com</t>
+        </is>
+      </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
           <t>https://htechconference.com</t>
@@ -1275,7 +1583,11 @@
           <t>https://www.linkedin.com/in/drjonathanleary</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>https://htechconference.com</t>
+        </is>
+      </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
           <t>https://htechconference.com</t>
@@ -1337,10 +1649,130 @@
           <t>https://www.linkedin.com/in/caseycaruso</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>https://htechconference.com</t>
+        </is>
+      </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
           <t>https://htechconference.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>"Built Different" - Calvario Men's Conference</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Gabby Mejia</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Calvario Church</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Speaker</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/built-different-calvario-mens-conference-registration-2001398535897</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>"Built Different" - Calvario Men's Conference</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Nehemias Santiago</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Calvario Church</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Speaker</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/built-different-calvario-mens-conference-registration-2001398535897</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>"Built Different" - Calvario Men's Conference</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Israel Martinez</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Calvario Church</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Speaker</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/built-different-calvario-mens-conference-registration-2001398535897</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>"Built Different" - Calvario Men's Conference</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Omar Johnson</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Calvario Church</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Speaker</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/built-different-calvario-mens-conference-registration-2001398535897</t>
         </is>
       </c>
     </row>
@@ -1355,18 +1787,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="72" customWidth="1" min="5" max="5"/>
+    <col width="82" customWidth="1" min="5" max="5"/>
     <col width="109" customWidth="1" min="6" max="6"/>
     <col width="72" customWidth="1" min="7" max="7"/>
     <col width="97" customWidth="1" min="8" max="8"/>
-    <col width="82" customWidth="1" min="9" max="9"/>
+    <col width="99" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1569,6 +2001,162 @@
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>https://www.fabtechexpo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-63D045</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>"Built Different" - Calvario Men's Conference</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Religion &amp; Spirituality</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>General Attendees</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/built-different-calvario-mens-conference-registration-2001398535897</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-5CCD8A</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Congress of Neurological Surgeons - CNS Annual Meeting</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cns.org/annualmeeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-310642</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>TEDxOshkosh 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Open to the Public</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>General Public, Innovators, Thinkers</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>https://TEDxOshkosh.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-D12D7F</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>ANEW Conference 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/anew-conference-2026-tickets-1998997596623</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix the linkedin details scrap
</commit_message>
<xml_diff>
--- a/data/excel/usa_conferences_published.xlsx
+++ b/data/excel/usa_conferences_published.xlsx
@@ -468,22 +468,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="57" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="69" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="51" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="73" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="99" customWidth="1" min="11" max="11"/>
-    <col width="99" customWidth="1" min="12" max="12"/>
-    <col width="99" customWidth="1" min="13" max="13"/>
+    <col width="115" customWidth="1" min="11" max="11"/>
+    <col width="116" customWidth="1" min="12" max="12"/>
+    <col width="115" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -1130,6 +1130,582 @@
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-AAD5AF</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>PRAISE BY THE WAVES 10th ANNUAL CONFERENCE:  APPOINTED FOR THIS</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>BWI Airport Marriott</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Praise by the Waves</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/praise-by-the-waves-10th-annual-conference-appointed-for-this-tickets-1996805798897</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/praise-by-the-waves-10th-annual-conference-appointed-for-this-tickets-1996805798897</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/praise-by-the-waves-10th-annual-conference-appointed-for-this-tickets-1996805798897</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-24BF68</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>American Public Health Association - APHA</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Henry B</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Tsnn</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>http://www.apha.org/events-and-meetings/annual</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>http://www.apha.org/events-and-meetings/annual</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>http://www.apha.org/events-and-meetings/annual</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-794BE4</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>San Diego Bay Wine + Food Festival</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>San Diego, CA, United States</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Tsnn</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sandiegowineclassic.com/</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sandiegowineclassic.com/</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sandiegowineclassic.com/</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-F9EF92</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Wisconsin Lodging Trade Show - WHLA</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Kalahari Resort &amp; Convention Center Wisconsin Dells, WI, United States</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Tsnn</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>https://web.wisconsinlodging.org/events/2026-Wisconsin-Lodging-Conference-Trade-Show-198/details</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>https://web.wisconsinlodging.org/events/2026-Wisconsin-Lodging-Conference-Trade-Show-198/details</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>https://web.wisconsinlodging.org/events/2026-Wisconsin-Lodging-Conference-Trade-Show-198/details</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-06CF74</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Melanin Medicine: Breath, Sound, &amp; Therapy</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Medicines &amp; Hospitals / Technology</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>First United Methodist Church of Germantown FUMCOG</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>HealYourLovePeriod</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/melanin-medicine-breath-sound-therapy-tickets-2003609520010</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/melanin-medicine-breath-sound-therapy-tickets-2003609520010</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/melanin-medicine-breath-sound-therapy-tickets-2003609520010</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-0A0052</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>PHILADELPHIA  PRO CONFERENCE</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>The Desmond Hotel - Malvern</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>National Aesthetic Spa Network (NASNPRO)</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>https://thebonnerinstitute.com/</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/philadelphia-pro-conference-registration-1965475113975</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>https://thebonnerinstitute.com/</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-D128F5</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>THE FUTURE OF AI IN SPORTS, GAMES, ENTERTAINMENT &amp; CREATOR ECONOMY</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions / Financial Services / Technology</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Fairmont San Francisco</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Silicon Valley AI Roadshow</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>https://indina-consulting-innovation-lab.kit.com/ai-summit-2026</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/the-future-of-ai-in-sports-games-entertainment-creator-economy-tickets-2000775248628</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>https://indina-consulting-innovation-lab.kit.com/ai-summit-2026</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-FE1647</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>U.S.-India AI Business Summit 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>National India Hub</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/us-india-ai-business-summit-2026-tickets-1999307250807</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/us-india-ai-business-summit-2026-tickets-1999307250807</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/us-india-ai-business-summit-2026-tickets-1999307250807</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
@@ -1787,18 +2363,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="57" customWidth="1" min="2" max="2"/>
+    <col width="69" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="82" customWidth="1" min="5" max="5"/>
-    <col width="109" customWidth="1" min="6" max="6"/>
+    <col width="153" customWidth="1" min="5" max="5"/>
+    <col width="161" customWidth="1" min="6" max="6"/>
     <col width="72" customWidth="1" min="7" max="7"/>
-    <col width="97" customWidth="1" min="8" max="8"/>
-    <col width="99" customWidth="1" min="9" max="9"/>
+    <col width="184" customWidth="1" min="8" max="8"/>
+    <col width="115" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2157,6 +2733,318 @@
       <c r="I9" s="4" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/anew-conference-2026-tickets-1998997596623</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-AAD5AF</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>PRAISE BY THE WAVES 10th ANNUAL CONFERENCE:  APPOINTED FOR THIS</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/praise-by-the-waves-10th-annual-conference-appointed-for-this-tickets-1996805798897</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-F9EF92</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Wisconsin Lodging Trade Show - WHLA</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>https://web.wisconsinlodging.org/events/2026-Wisconsin-Lodging-Conference-Trade-Show-198/details</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-24BF68</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>American Public Health Association - APHA</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>http://www.apha.org/events-and-meetings/annual</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-794BE4</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>San Diego Bay Wine + Food Festival</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sandiegowineclassic.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-FE1647</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>U.S.-India AI Business Summit 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Enterprise AI / AI Solutions seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/us-india-ai-business-summit-2026-tickets-1999307250807</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-D128F5</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>THE FUTURE OF AI IN SPORTS, GAMES, ENTERTAINMENT &amp; CREATOR ECONOMY</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Financial Analysts, Banking Executives, FinTech Leaders, Investors; Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Enterprise AI / AI Solutions / Financial Services / Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AI / AI Solutions / Financial Services / Technology</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>CFOs, VP of Finance, Risk Managers, Compliance Officers, FinTech Developers; CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>https://indina-consulting-innovation-lab.kit.com/ai-summit-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-0A0052</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>PHILADELPHIA  PRO CONFERENCE</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>https://thebonnerinstitute.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>CONF-2026-06CF74</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Melanin Medicine: Breath, Sound, &amp; Therapy</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Healthcare Providers, Clinicians, Researchers, Health Tech Executives; Engineers, Architects, AI Practitioners, Technology Leaders, C-Suite Executives</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Professionals, leaders, and decision-makers in Medicines &amp; Hospitals / Technology seeking cutting-edge insights and collaboration.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Medicines &amp; Hospitals / Technology</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Chief Medical Officers, Physicians, Clinical Directors, Healthcare Administrators, Researchers; CTOs, CISOs, VP of Engineering, Data Scientists, AI Researchers, Solutions Architects</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/melanin-medicine-breath-sound-therapy-tickets-2003609520010</t>
         </is>
       </c>
     </row>
@@ -5668,10 +6556,14 @@
           <t>ABC</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/daymondjohn/</t>
+        </is>
+      </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr"/>
@@ -5688,7 +6580,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:15:15.654499</t>
+          <t>2026-10-30T07:09:41.167864</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
@@ -5731,7 +6623,7 @@
       <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr"/>
@@ -5748,7 +6640,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:15:17.070209</t>
+          <t>2026-10-30T07:09:32.533504</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
@@ -5788,10 +6680,14 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/willgrannis</t>
+        </is>
+      </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr"/>
@@ -5808,7 +6704,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:15:18.214775</t>
+          <t>2026-10-30T07:09:43.372731</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
@@ -5851,7 +6747,7 @@
       <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr"/>
@@ -5868,7 +6764,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:15:19.415434</t>
+          <t>2026-10-30T07:09:34.667878</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -5908,10 +6804,14 @@
           <t>ServiceNow</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/paulfipps/</t>
+        </is>
+      </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr"/>
@@ -5928,7 +6828,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:15:20.557932</t>
+          <t>2026-10-30T07:09:35.224802</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
@@ -5968,10 +6868,14 @@
           <t>Uber</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/sachinkansal</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr"/>
@@ -5988,7 +6892,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:15:21.761452</t>
+          <t>2026-10-30T07:09:37.447287</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -6028,10 +6932,14 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/majid-mohammed-abdul-767a1440/</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr"/>
@@ -6048,7 +6956,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:17:12.595684</t>
+          <t>2026-10-30T07:09:38.994674</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -6088,10 +6996,14 @@
           <t>Waze</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alex-ohayon-79174665</t>
+        </is>
+      </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr"/>
@@ -6108,7 +7020,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:17:13.916975</t>
+          <t>2026-10-30T07:10:07.762937</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
@@ -6148,10 +7060,14 @@
           <t>Credit Karma</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ashir-alam</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr"/>
@@ -6168,7 +7084,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:17:15.134454</t>
+          <t>2026-10-30T07:10:10.126475</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
@@ -6208,10 +7124,14 @@
           <t>Uber</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/piyushmaheshwari1</t>
+        </is>
+      </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr"/>
@@ -6228,7 +7148,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:17:16.373663</t>
+          <t>2026-10-30T07:09:45.352326</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
@@ -6268,10 +7188,14 @@
           <t>ABNAMRO Bank</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ramzialashabi/</t>
+        </is>
+      </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
@@ -6288,7 +7212,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:17:17.533131</t>
+          <t>2026-10-30T07:09:46.968659</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
@@ -6328,10 +7252,14 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sean-bjurstrom/</t>
+        </is>
+      </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
@@ -6348,7 +7276,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:17:18.843216</t>
+          <t>2026-10-30T07:09:49.223020</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
@@ -6388,10 +7316,14 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sneha-rao/</t>
+        </is>
+      </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr"/>
@@ -6408,7 +7340,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:17:20.135742</t>
+          <t>2026-10-30T07:09:51.060120</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
@@ -6448,10 +7380,14 @@
           <t>Notion</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/yunhao-qing/</t>
+        </is>
+      </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr"/>
@@ -6468,7 +7404,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:17:21.313398</t>
+          <t>2026-10-30T07:09:52.856491</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
@@ -6511,7 +7447,7 @@
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr"/>
@@ -6528,7 +7464,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.757504</t>
+          <t>2026-10-30T07:10:13.508619</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
@@ -6571,7 +7507,7 @@
       <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr"/>
@@ -6588,7 +7524,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.758119</t>
+          <t>2026-10-30T07:09:55.095376</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
@@ -6628,10 +7564,14 @@
           <t>Samsung Ventures</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jihong-kim-a6696aa/</t>
+        </is>
+      </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr"/>
@@ -6648,7 +7588,7 @@
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.758563</t>
+          <t>2026-10-30T07:09:55.633282</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
@@ -6688,10 +7628,14 @@
           <t>Khosla Ventures</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rajesh-swaminathan-960a501/</t>
+        </is>
+      </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr"/>
@@ -6708,7 +7652,7 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.759025</t>
+          <t>2026-10-30T07:09:57.874677</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
@@ -6751,7 +7695,7 @@
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr"/>
@@ -6768,7 +7712,7 @@
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.759322</t>
+          <t>2026-10-30T07:10:15.563037</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
@@ -6808,10 +7752,14 @@
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/melanie-nakagawa-2781505/</t>
+        </is>
+      </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr"/>
@@ -6828,7 +7776,7 @@
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.759689</t>
+          <t>2026-10-30T07:09:59.969329</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
@@ -6868,10 +7816,14 @@
           <t>Uber</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sachinkansal/</t>
+        </is>
+      </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr"/>
@@ -6888,7 +7840,7 @@
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.760185</t>
+          <t>2026-10-30T07:10:01.907811</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -6928,10 +7880,14 @@
           <t>Norwest Partners</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/scottbeechuk/</t>
+        </is>
+      </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr"/>
@@ -6948,7 +7904,7 @@
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.760554</t>
+          <t>2026-10-30T07:10:03.870798</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -6988,10 +7944,14 @@
           <t>Foundation Capital</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jayagupta10/</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr"/>
@@ -7008,7 +7968,7 @@
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:19:40.760975</t>
+          <t>2026-10-30T07:10:05.198728</t>
         </is>
       </c>
       <c r="N24" s="4" t="inlineStr">
@@ -7048,10 +8008,14 @@
           <t>Rainforest Distribution</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/amaury-schoon-42bb5235/</t>
+        </is>
+      </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr"/>
@@ -7068,7 +8032,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:30.195024</t>
+          <t>2026-10-30T07:10:16.098827</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -7108,10 +8072,14 @@
           <t>Rainforest Distribution</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jimmy-sebbah-5b8b8825/</t>
+        </is>
+      </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr"/>
@@ -7128,7 +8096,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:31.476476</t>
+          <t>2026-10-30T07:10:18.096222</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -7168,10 +8136,14 @@
           <t>Whole Foods Market</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/johnlawson2007/</t>
+        </is>
+      </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr"/>
@@ -7188,7 +8160,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:32.766731</t>
+          <t>2026-10-30T07:10:20.313172</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -7228,10 +8200,14 @@
           <t>The Goods Mart</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rachelkrupa/</t>
+        </is>
+      </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr"/>
@@ -7248,7 +8224,7 @@
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:34.133782</t>
+          <t>2026-10-30T07:10:22.031831</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
@@ -7288,10 +8264,14 @@
           <t>America's Food Basket</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/javier-intriago-valle/</t>
+        </is>
+      </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr"/>
@@ -7308,7 +8288,7 @@
       </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:35.371194</t>
+          <t>2026-10-30T07:10:24.539011</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr">
@@ -7348,10 +8328,14 @@
           <t>Naturally Good Foods and Cafe</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/lkkatz/</t>
+        </is>
+      </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr"/>
@@ -7368,7 +8352,7 @@
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:36.474834</t>
+          <t>2026-10-30T07:10:26.449327</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
@@ -7408,10 +8392,14 @@
           <t>FreshDirect</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/juliangoncalves/</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr"/>
@@ -7428,7 +8416,7 @@
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:37.575419</t>
+          <t>2026-10-30T07:10:28.016165</t>
         </is>
       </c>
       <c r="N31" s="4" t="inlineStr">
@@ -7468,10 +8456,14 @@
           <t>Condé Nast</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/oliviatarantino/</t>
+        </is>
+      </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr"/>
@@ -7488,7 +8480,7 @@
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:38.905780</t>
+          <t>2026-10-30T07:10:29.645084</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
@@ -7528,10 +8520,14 @@
           <t>Wakefern</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/glenn-cunningham-5799b979/</t>
+        </is>
+      </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr"/>
@@ -7548,7 +8544,7 @@
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:39.965897</t>
+          <t>2026-10-30T07:11:00.988800</t>
         </is>
       </c>
       <c r="N33" s="4" t="inlineStr">
@@ -7588,10 +8584,14 @@
           <t>Wakefern</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/fedele-stella-7a0447265/</t>
+        </is>
+      </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr"/>
@@ -7608,7 +8608,7 @@
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:41.091624</t>
+          <t>2026-10-30T07:10:33.109667</t>
         </is>
       </c>
       <c r="N34" s="4" t="inlineStr">
@@ -7648,10 +8648,14 @@
           <t>Imaginary Ventures</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tara-campbell-7ba18946/</t>
+        </is>
+      </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr"/>
@@ -7668,7 +8672,7 @@
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:42.457222</t>
+          <t>2026-10-30T07:10:37.002145</t>
         </is>
       </c>
       <c r="N35" s="4" t="inlineStr">
@@ -7708,10 +8712,14 @@
           <t>Mondelēz International</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/lsafran/</t>
+        </is>
+      </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr"/>
@@ -7728,7 +8736,7 @@
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:43.610877</t>
+          <t>2026-10-30T07:10:38.549489</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -7768,10 +8776,14 @@
           <t>Vanterra Ventures</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/elizabeth-yang-02/</t>
+        </is>
+      </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr"/>
@@ -7788,7 +8800,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:44.852953</t>
+          <t>2026-10-30T07:10:40.497259</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -7828,10 +8840,14 @@
           <t>Wakefern</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tanya-seber-b3a660a1/</t>
+        </is>
+      </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr"/>
@@ -7848,7 +8864,7 @@
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:46.017023</t>
+          <t>2026-10-30T07:10:43.335695</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
@@ -7888,10 +8904,14 @@
           <t>Alumni Ventures</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bozhena-k/</t>
+        </is>
+      </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr"/>
@@ -7908,7 +8928,7 @@
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:47.204364</t>
+          <t>2026-10-30T07:10:45.424282</t>
         </is>
       </c>
       <c r="N39" s="4" t="inlineStr">
@@ -7948,10 +8968,14 @@
           <t>Great Circle Ventures</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ryanperry4</t>
+        </is>
+      </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr"/>
@@ -7968,7 +8992,7 @@
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:48.615584</t>
+          <t>2026-10-30T07:11:29.453094</t>
         </is>
       </c>
       <c r="N40" s="4" t="inlineStr">
@@ -8008,10 +9032,14 @@
           <t>Farm to People</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bradyroger/</t>
+        </is>
+      </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr"/>
@@ -8028,7 +9056,7 @@
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:50.009397</t>
+          <t>2026-10-30T07:10:47.600706</t>
         </is>
       </c>
       <c r="N41" s="4" t="inlineStr">
@@ -8071,7 +9099,7 @@
       <c r="G42" s="4" t="inlineStr"/>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr"/>
@@ -8088,7 +9116,7 @@
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:51.262998</t>
+          <t>2026-10-30T07:10:51.273610</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
@@ -8128,10 +9156,14 @@
           <t>Sling Ventures</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/brandonalster/</t>
+        </is>
+      </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr"/>
@@ -8148,7 +9180,7 @@
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:52.623233</t>
+          <t>2026-10-30T07:10:53.357296</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -8191,7 +9223,7 @@
       <c r="G44" s="4" t="inlineStr"/>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr"/>
@@ -8208,7 +9240,7 @@
       </c>
       <c r="M44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:54.022497</t>
+          <t>2026-10-30T07:10:57.069711</t>
         </is>
       </c>
       <c r="N44" s="4" t="inlineStr">
@@ -8248,10 +9280,14 @@
           <t>FreshDirect</t>
         </is>
       </c>
-      <c r="G45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/katherine-andrew/</t>
+        </is>
+      </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr"/>
@@ -8268,7 +9304,7 @@
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:55.444807</t>
+          <t>2026-10-30T07:11:02.706846</t>
         </is>
       </c>
       <c r="N45" s="4" t="inlineStr">
@@ -8308,10 +9344,14 @@
           <t>FreshDirect</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/elsemieke-vriend-112435124/</t>
+        </is>
+      </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr"/>
@@ -8328,7 +9368,7 @@
       </c>
       <c r="M46" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:56.856912</t>
+          <t>2026-10-30T07:10:58.890868</t>
         </is>
       </c>
       <c r="N46" s="4" t="inlineStr">
@@ -8368,10 +9408,14 @@
           <t>FreshDirect</t>
         </is>
       </c>
-      <c r="G47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/fatoumatabarry-/</t>
+        </is>
+      </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr"/>
@@ -8388,7 +9432,7 @@
       </c>
       <c r="M47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:58.143774</t>
+          <t>2026-10-30T07:11:04.751386</t>
         </is>
       </c>
       <c r="N47" s="4" t="inlineStr">
@@ -8428,10 +9472,14 @@
           <t>Manna Tree Partners</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/graceverrier/</t>
+        </is>
+      </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr"/>
@@ -8448,7 +9496,7 @@
       </c>
       <c r="M48" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:24:59.249691</t>
+          <t>2026-10-30T07:11:06.429506</t>
         </is>
       </c>
       <c r="N48" s="4" t="inlineStr">
@@ -8491,7 +9539,7 @@
       <c r="G49" s="4" t="inlineStr"/>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr"/>
@@ -8508,7 +9556,7 @@
       </c>
       <c r="M49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:25:00.684946</t>
+          <t>2026-10-30T07:11:10.849340</t>
         </is>
       </c>
       <c r="N49" s="4" t="inlineStr">
@@ -8548,10 +9596,14 @@
           <t>Alumni Ventures</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/charlotte-jenkins-/</t>
+        </is>
+      </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr"/>
@@ -8568,7 +9620,7 @@
       </c>
       <c r="M50" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:25:02.029117</t>
+          <t>2026-10-30T07:11:12.492848</t>
         </is>
       </c>
       <c r="N50" s="4" t="inlineStr">
@@ -8608,10 +9660,14 @@
           <t>Pep</t>
         </is>
       </c>
-      <c r="G51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/abbygiannuzzi/</t>
+        </is>
+      </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr"/>
@@ -8628,7 +9684,7 @@
       </c>
       <c r="M51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:25:03.279832</t>
+          <t>2026-10-30T07:11:14.604658</t>
         </is>
       </c>
       <c r="N51" s="4" t="inlineStr">
@@ -8668,10 +9724,14 @@
           <t>The Wealth Mosaic</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr"/>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michael-partnow/</t>
+        </is>
+      </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr"/>
@@ -8688,7 +9748,7 @@
       </c>
       <c r="M52" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T11:25:32.612985</t>
+          <t>2026-10-30T07:11:16.695848</t>
         </is>
       </c>
       <c r="N52" s="4" t="inlineStr">
@@ -8728,10 +9788,14 @@
           <t>BCA</t>
         </is>
       </c>
-      <c r="G53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/haryantobudiman/</t>
+        </is>
+      </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr"/>
@@ -8748,7 +9812,7 @@
       </c>
       <c r="M53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T12:07:07.040784</t>
+          <t>2026-10-30T07:11:18.574526</t>
         </is>
       </c>
       <c r="N53" s="4" t="inlineStr">
@@ -8788,10 +9852,14 @@
           <t>Capital Group</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr"/>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/winnie-kwan-30588151/</t>
+        </is>
+      </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr"/>
@@ -8808,7 +9876,7 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T12:07:08.151360</t>
+          <t>2026-10-30T07:11:22.129101</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
@@ -8848,10 +9916,14 @@
           <t>KPS Capital Partners Asia</t>
         </is>
       </c>
-      <c r="G55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/takahiroishikawa/</t>
+        </is>
+      </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr"/>
@@ -8868,7 +9940,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T12:07:10.987027</t>
+          <t>2026-10-30T07:11:24.084319</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -8908,10 +9980,14 @@
           <t>SKIMS</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr"/>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tracynguyenca/</t>
+        </is>
+      </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I56" s="4" t="inlineStr"/>
@@ -8928,7 +10004,7 @@
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>2026-10-29T12:07:12.145269</t>
+          <t>2026-10-30T07:11:26.767686</t>
         </is>
       </c>
       <c r="N56" s="4" t="inlineStr">

</xml_diff>